<commit_message>
docs: complete business discovery and prepare for solution architecture
</commit_message>
<xml_diff>
--- a/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
+++ b/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd01d60e8fdc72b3/Projects/Construction_Analytics_Platform/Documentation/Formal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F6A6E23-2737-4ABE-889A-135D794CF9EA}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CA9293E-A78C-423C-A30A-3031B9198EF1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" activeTab="5" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
+    <workbookView minimized="1" xWindow="6165" yWindow="1290" windowWidth="21600" windowHeight="11430" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
   </bookViews>
   <sheets>
     <sheet name="Business Discoveries" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="216">
   <si>
     <t>Business Question</t>
   </si>
@@ -410,13 +410,295 @@
   </si>
   <si>
     <t>Units completed per labor hour or shift for a specific activity.</t>
+  </si>
+  <si>
+    <t>BD-301</t>
+  </si>
+  <si>
+    <t>BD-302</t>
+  </si>
+  <si>
+    <t>BD-303</t>
+  </si>
+  <si>
+    <t>BD-304</t>
+  </si>
+  <si>
+    <t>BD-305</t>
+  </si>
+  <si>
+    <t>BD-306</t>
+  </si>
+  <si>
+    <t>BD-307</t>
+  </si>
+  <si>
+    <t>BD-308</t>
+  </si>
+  <si>
+    <t>BD-309</t>
+  </si>
+  <si>
+    <t>BD-310</t>
+  </si>
+  <si>
+    <t>BD-311</t>
+  </si>
+  <si>
+    <t>Financial Data Validation</t>
+  </si>
+  <si>
+    <t>Job Cost validates operational postings before financial reporting.</t>
+  </si>
+  <si>
+    <t>Improves financial accuracy.</t>
+  </si>
+  <si>
+    <t>Exception reporting required.</t>
+  </si>
+  <si>
+    <t>Forecasting</t>
+  </si>
+  <si>
+    <t>Management relies on forecasted performance to support decision-making.</t>
+  </si>
+  <si>
+    <t>Forecast KPIs required.</t>
+  </si>
+  <si>
+    <t>Early Budget Adjustments</t>
+  </si>
+  <si>
+    <t>Budget changes should occur as soon as new information becomes available.</t>
+  </si>
+  <si>
+    <t>Improves financial visibility.</t>
+  </si>
+  <si>
+    <t>Budget revision history required.</t>
+  </si>
+  <si>
+    <t>Closed Job Reviews</t>
+  </si>
+  <si>
+    <t>Weekly reviews identify lessons learned from completed projects.</t>
+  </si>
+  <si>
+    <t>Supports continuous improvement.</t>
+  </si>
+  <si>
+    <t>Closed Job Review dashboard.</t>
+  </si>
+  <si>
+    <t>Labor Recovery</t>
+  </si>
+  <si>
+    <t>Labor utilization directly influences burden recovery.</t>
+  </si>
+  <si>
+    <t>Labor efficiency affects profitability.</t>
+  </si>
+  <si>
+    <t>Labor recovery analytics.</t>
+  </si>
+  <si>
+    <t>Equipment Recovery</t>
+  </si>
+  <si>
+    <t>Equipment utilization influences equipment cost recovery.</t>
+  </si>
+  <si>
+    <t>Equipment performance affects profitability.</t>
+  </si>
+  <si>
+    <t>Equipment utilization KPIs.</t>
+  </si>
+  <si>
+    <t>Executive Scorecard</t>
+  </si>
+  <si>
+    <t>WIP functions as the primary executive performance scorecard.</t>
+  </si>
+  <si>
+    <t>Supports executive decision-making.</t>
+  </si>
+  <si>
+    <t>Executive Performance dashboard.</t>
+  </si>
+  <si>
+    <t>Remaining Budget</t>
+  </si>
+  <si>
+    <t>Remaining budget and remaining scope determine project health.</t>
+  </si>
+  <si>
+    <t>Improves forecasting.</t>
+  </si>
+  <si>
+    <t>Project Health KPI.</t>
+  </si>
+  <si>
+    <t>Variance Thresholds</t>
+  </si>
+  <si>
+    <t>Significant project variances should trigger detailed management review.</t>
+  </si>
+  <si>
+    <t>Focuses attention on high-risk projects.</t>
+  </si>
+  <si>
+    <t>Configurable variance alerts.</t>
+  </si>
+  <si>
+    <t>Multi-Period Performance</t>
+  </si>
+  <si>
+    <t>Management simultaneously evaluates planned, current, historical, and forecast performance.</t>
+  </si>
+  <si>
+    <t>Encourages balanced decision-making.</t>
+  </si>
+  <si>
+    <t>Time-based analytics model.</t>
+  </si>
+  <si>
+    <t>Role-Based Reporting</t>
+  </si>
+  <si>
+    <t>Reports should be filtered according to organizational responsibility.</t>
+  </si>
+  <si>
+    <t>Improves relevance and usability.</t>
+  </si>
+  <si>
+    <t>Row-level security and filtered dashboards.</t>
+  </si>
+  <si>
+    <t>BD-401</t>
+  </si>
+  <si>
+    <t>BD-402</t>
+  </si>
+  <si>
+    <t>BD-403</t>
+  </si>
+  <si>
+    <t>BD-404</t>
+  </si>
+  <si>
+    <t>BD-405</t>
+  </si>
+  <si>
+    <t>BD-406</t>
+  </si>
+  <si>
+    <t>BD-407</t>
+  </si>
+  <si>
+    <t>BD-408</t>
+  </si>
+  <si>
+    <t>Customer Relationships Influence Pricing Strategy</t>
+  </si>
+  <si>
+    <t>Approximately 80–85% of annual work is awarded to repeat customers. Pricing decisions consider customer relationships, service expectations, location, and project type in addition to project costs.</t>
+  </si>
+  <si>
+    <t>Estimating is influenced by both financial and strategic business considerations.</t>
+  </si>
+  <si>
+    <t>The solution should preserve customer, sales representative, and historical project information to support relationship-based analysis.</t>
+  </si>
+  <si>
+    <t>Estimating Defines the Project Execution Plan</t>
+  </si>
+  <si>
+    <t>The estimating process establishes the expected crew, equipment, production rates, material quantities, suppliers, project margin, and operational approach before work begins.</t>
+  </si>
+  <si>
+    <t>The estimate becomes the operational blueprint for project execution.</t>
+  </si>
+  <si>
+    <t>The database should capture operational planning information as part of the estimating and budgeting process.</t>
+  </si>
+  <si>
+    <t>Production Standards Combine Historical Data and Professional Judgment</t>
+  </si>
+  <si>
+    <t>Production rates are developed using historical production data, estimator experience, superintendent knowledge, crew capability, and project-specific conditions.</t>
+  </si>
+  <si>
+    <t>Production expectations cannot rely solely on historical averages and require professional judgment.</t>
+  </si>
+  <si>
+    <t>Production standards should support configurable values that can be adjusted based on project characteristics.</t>
+  </si>
+  <si>
+    <t>Standard Crew Configurations Improve Estimating Consistency</t>
+  </si>
+  <si>
+    <t>Most construction activities are performed using predefined crew configurations with standard equipment packages. Project-specific adjustments are made only when required.</t>
+  </si>
+  <si>
+    <t>Standardization improves estimating consistency while maintaining flexibility for unique projects.</t>
+  </si>
+  <si>
+    <t>Standard crew and equipment templates should be modeled as reusable reference data.</t>
+  </si>
+  <si>
+    <t>Material Estimating Uses Different Methods Based on Material Type</t>
+  </si>
+  <si>
+    <t>Major construction materials are estimated using project-specific quantities and current supplier pricing, while incidental materials are estimated using historical usage factors.</t>
+  </si>
+  <si>
+    <t>Different estimating methodologies are required depending on the significance of the material.</t>
+  </si>
+  <si>
+    <t>The solution should distinguish between quantity-based major materials and allowance-based incidental materials.</t>
+  </si>
+  <si>
+    <t>Approved Estimates Become the Official Job Budget</t>
+  </si>
+  <si>
+    <t>Before work begins, the original estimate is reviewed, adjusted for scope changes, and normalized so each budget line reflects the project's approved gross margin. This reviewed estimate becomes the official job budget.</t>
+  </si>
+  <si>
+    <t>The approved budget becomes the baseline used throughout project execution and performance reporting.</t>
+  </si>
+  <si>
+    <t>The solution should preserve the relationship between the original estimate and the approved operational budget while maintaining budget revision history.</t>
+  </si>
+  <si>
+    <t>Project Handoff Provides a Common Operational Plan</t>
+  </si>
+  <si>
+    <t>After project award, the proposal, job budget, diagrams, and project notes are distributed to Project Managers, Superintendents, Foremen, and Project Coordinators.</t>
+  </si>
+  <si>
+    <t>All project stakeholders begin execution using the same operational information and expectations.</t>
+  </si>
+  <si>
+    <t>The solution should support centralized project documentation and role-based access to planning information.</t>
+  </si>
+  <si>
+    <t>Travel Is a Planned Component of Production</t>
+  </si>
+  <si>
+    <t>Travel time is estimated based on mobilization requirements and expected production hours and is budgeted and tracked separately from production activities.</t>
+  </si>
+  <si>
+    <t>Travel directly affects labor utilization, scheduling, and project profitability and should be managed independently.</t>
+  </si>
+  <si>
+    <t>Travel should remain a distinct project phase within the data model and analytics to support labor utilization and operational performance reporting.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -428,6 +710,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -462,7 +750,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -471,8 +759,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -807,8 +1111,765 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F02528A-58D3-45D6-A9F7-646AA94A3C40}">
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="198.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="104.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="141.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E2E8FE-B991-49FD-941C-2282A5D8D908}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="17.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
@@ -820,325 +1881,6 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E2E8FE-B991-49FD-941C-2282A5D8D908}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="17.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="98.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="17.42578125" style="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
docs: complete SA-001 business entity identification
</commit_message>
<xml_diff>
--- a/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
+++ b/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd01d60e8fdc72b3/Projects/Construction_Analytics_Platform/Documentation/Formal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="129" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CA9293E-A78C-423C-A30A-3031B9198EF1}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7B2EDD0-D692-4983-8B36-B6B0F89F2AF8}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="6165" yWindow="1290" windowWidth="21600" windowHeight="11430" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" activeTab="2" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
   </bookViews>
   <sheets>
     <sheet name="Business Discoveries" sheetId="1" r:id="rId1"/>
@@ -44,13 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="216">
-  <si>
-    <t>Business Question</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="299">
   <si>
     <t>KPI</t>
   </si>
@@ -94,15 +88,6 @@
     <t>Solution Impact</t>
   </si>
   <si>
-    <t>BQ ID</t>
-  </si>
-  <si>
-    <t>Related BD</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
     <t>Workshop</t>
   </si>
   <si>
@@ -692,6 +677,270 @@
   </si>
   <si>
     <t>Travel should remain a distinct project phase within the data model and analytics to support labor utilization and operational performance reporting.</t>
+  </si>
+  <si>
+    <t>FR ID</t>
+  </si>
+  <si>
+    <t>Requirement Title</t>
+  </si>
+  <si>
+    <t>Functional Requirement</t>
+  </si>
+  <si>
+    <t>FR-001</t>
+  </si>
+  <si>
+    <t>Customer and Site Separation</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Customer and Property/Site as separate entities and associate each job with exactly one customer and one site.</t>
+  </si>
+  <si>
+    <t>SA-001</t>
+  </si>
+  <si>
+    <t>FR-002</t>
+  </si>
+  <si>
+    <t>Opportunity-to-Job Traceability</t>
+  </si>
+  <si>
+    <t>The solution shall preserve traceability among opportunities, quotes, bid budgets, accepted scope, jobs, and original job budgets.</t>
+  </si>
+  <si>
+    <t>FR-003</t>
+  </si>
+  <si>
+    <t>Original Budget Preservation</t>
+  </si>
+  <si>
+    <t>The solution shall preserve the original job budget and calculate revised and adjusted budgets without overwriting original values.</t>
+  </si>
+  <si>
+    <t>FR-004</t>
+  </si>
+  <si>
+    <t>Change-Order Budgets</t>
+  </si>
+  <si>
+    <t>The solution shall maintain a separate budget for each change order and include only accepted change-order budgets in revised job analysis.</t>
+  </si>
+  <si>
+    <t>FR-005</t>
+  </si>
+  <si>
+    <t>Warranty Budgets</t>
+  </si>
+  <si>
+    <t>The solution shall support separate zero-revenue warranty budgets associated with the original job, cost codes, and warranty phases.</t>
+  </si>
+  <si>
+    <t>FR-006</t>
+  </si>
+  <si>
+    <t>Budget Adjustments</t>
+  </si>
+  <si>
+    <t>The solution shall support positive and negative quantity or cost adjustments while retaining adjustment date, value, reason, entered by, and notes.</t>
+  </si>
+  <si>
+    <t>FR-007</t>
+  </si>
+  <si>
+    <t>Revenue Restrictions</t>
+  </si>
+  <si>
+    <t>The solution shall permit revenue only through original and accepted change-order budgets and shall prevent ordinary cost adjustments from changing revenue.</t>
+  </si>
+  <si>
+    <t>FR-008</t>
+  </si>
+  <si>
+    <t>Job Responsibility Assignments</t>
+  </si>
+  <si>
+    <t>The solution shall support job-level PM, superintendent, sales, and estimator assignments and cost-code-level foreman assignments.</t>
+  </si>
+  <si>
+    <t>FR-009</t>
+  </si>
+  <si>
+    <t>Employee Time Detail</t>
+  </si>
+  <si>
+    <t>The solution shall capture employee time by date, job, cost code, phase, labor code, hours, start time, and end time.</t>
+  </si>
+  <si>
+    <t>FR-010</t>
+  </si>
+  <si>
+    <t>Prevailing-Wage Rates</t>
+  </si>
+  <si>
+    <t>The solution shall support effective-dated prevailing-wage rates by labor classification and apply the higher of the regular or prevailing rate.</t>
+  </si>
+  <si>
+    <t>FR-011</t>
+  </si>
+  <si>
+    <t>Separate Burden Cost</t>
+  </si>
+  <si>
+    <t>The solution shall maintain burden as a separate cost type and distinguish tax burden from indirect burden.</t>
+  </si>
+  <si>
+    <t>FR-012</t>
+  </si>
+  <si>
+    <t>Equipment Unit Tracking</t>
+  </si>
+  <si>
+    <t>The solution shall track individual equipment units, effective-dated rates, daily usage, calculated hours, and calculated cost.</t>
+  </si>
+  <si>
+    <t>FR-013</t>
+  </si>
+  <si>
+    <t>Equipment Utilization Standards</t>
+  </si>
+  <si>
+    <t>The solution shall calculate equipment hours using applicable crew shift hours and effective-dated division utilization factors.</t>
+  </si>
+  <si>
+    <t>FR-014</t>
+  </si>
+  <si>
+    <t>Inventory Average Cost</t>
+  </si>
+  <si>
+    <t>The solution shall apply the inventory average cost in effect when material is issued and preserve the applied historical unit cost.</t>
+  </si>
+  <si>
+    <t>FR-015</t>
+  </si>
+  <si>
+    <t>Purchased Material Reconciliation</t>
+  </si>
+  <si>
+    <t>The solution shall retain foreman-reported, supplier-ticket, and invoiced material quantities as separate values.</t>
+  </si>
+  <si>
+    <t>FR-016</t>
+  </si>
+  <si>
+    <t>Purchase-Order Control</t>
+  </si>
+  <si>
+    <t>The solution shall restrict each purchase order to one job and one vendor while permitting multiple cost codes, phases, and items.</t>
+  </si>
+  <si>
+    <t>FR-017</t>
+  </si>
+  <si>
+    <t>Commitment Reporting</t>
+  </si>
+  <si>
+    <t>The solution shall calculate committed cost from open purchase orders through the selected reporting cutoff date.</t>
+  </si>
+  <si>
+    <t>FR-018</t>
+  </si>
+  <si>
+    <t>Detailed Job-Cost Transactions</t>
+  </si>
+  <si>
+    <t>The solution shall retain individual job-cost line items and support drill-through from totals to source transactions.</t>
+  </si>
+  <si>
+    <t>FR-019</t>
+  </si>
+  <si>
+    <t>Date-Used Reporting</t>
+  </si>
+  <si>
+    <t>The solution shall attribute operational and financial cost analysis to the date the resource or cost was used.</t>
+  </si>
+  <si>
+    <t>FR-020</t>
+  </si>
+  <si>
+    <t>Transaction Audit Trail</t>
+  </si>
+  <si>
+    <t>The solution shall preserve original, reversal, and corrected transactions and their relationships.</t>
+  </si>
+  <si>
+    <t>FR-021</t>
+  </si>
+  <si>
+    <t>WIP Calculation</t>
+  </si>
+  <si>
+    <t>The solution shall calculate cost-to-cost percent complete and cap earned revenue at revised contract revenue.</t>
+  </si>
+  <si>
+    <t>FR-022</t>
+  </si>
+  <si>
+    <t>Job Forecast</t>
+  </si>
+  <si>
+    <t>The solution shall calculate forecast final cost using actual cost, open commitments, and remaining to spend.</t>
+  </si>
+  <si>
+    <t>FR-023</t>
+  </si>
+  <si>
+    <t>Fade and Gain</t>
+  </si>
+  <si>
+    <t>The solution shall calculate fade or gain as adjusted budgeted cost minus actual cost.</t>
+  </si>
+  <si>
+    <t>FR-024</t>
+  </si>
+  <si>
+    <t>Job Billing</t>
+  </si>
+  <si>
+    <t>The solution shall associate each customer invoice with one job and calculate billed revenue to date at the job level.</t>
+  </si>
+  <si>
+    <t>FR-025</t>
+  </si>
+  <si>
+    <t>Job Lifecycle Control</t>
+  </si>
+  <si>
+    <t>The solution shall distinguish Awarded, In Progress, Complete, Closed, and Cancelled jobs and require reopening before posting to a closed job.</t>
+  </si>
+  <si>
+    <t>FR-026</t>
+  </si>
+  <si>
+    <t>Standard Cost Hierarchy</t>
+  </si>
+  <si>
+    <t>The solution shall use Job → Cost Code → Phase → Cost Type across budgets and actual job-cost transactions.</t>
+  </si>
+  <si>
+    <t>FR-027</t>
+  </si>
+  <si>
+    <t>Valid Posting Combinations</t>
+  </si>
+  <si>
+    <t>The solution shall permit posting only to cost codes and phases activated for the job.</t>
+  </si>
+  <si>
+    <t>FR-028</t>
+  </si>
+  <si>
+    <t>Standard Cost Types</t>
+  </si>
+  <si>
+    <t>The solution shall support L, B, G, M, E, S, and Z as the standard company cost types.</t>
   </si>
 </sst>
 </file>
@@ -750,7 +999,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -774,9 +1023,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1126,738 +1376,738 @@
   <sheetData>
     <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="F1" s="5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="G2" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>45</v>
-      </c>
       <c r="G5" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>66</v>
-      </c>
       <c r="G9" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B24" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="B26" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="B27" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="B28" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F24" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
+      <c r="B29" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
+      <c r="B30" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="B31" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="E30" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="E32" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1882,301 +2132,301 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="F1" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="G2" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="G5" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="G9" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -2186,31 +2436,508 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{979FD651-F2D4-4BEE-84B1-39B645FFAE94}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.85546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="145.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>4</v>
+      <c r="E1" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -2231,58 +2958,58 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -2304,121 +3031,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2437,58 +3164,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete SA-002 entity relationship definition
</commit_message>
<xml_diff>
--- a/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
+++ b/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd01d60e8fdc72b3/Projects/Construction_Analytics_Platform/Documentation/Formal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="134" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7B2EDD0-D692-4983-8B36-B6B0F89F2AF8}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FAD9689-C9EA-4C39-AF0C-C98BC151269C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" activeTab="2" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="438">
   <si>
     <t>KPI</t>
   </si>
@@ -691,12 +691,6 @@
     <t>FR-001</t>
   </si>
   <si>
-    <t>Customer and Site Separation</t>
-  </si>
-  <si>
-    <t>The solution shall maintain Customer and Property/Site as separate entities and associate each job with exactly one customer and one site.</t>
-  </si>
-  <si>
     <t>SA-001</t>
   </si>
   <si>
@@ -941,6 +935,429 @@
   </si>
   <si>
     <t>The solution shall support L, B, G, M, E, S, and Z as the standard company cost types.</t>
+  </si>
+  <si>
+    <t>Customer and Site Information</t>
+  </si>
+  <si>
+    <t>The solution shall associate each opportunity and job with exactly one customer and one site while storing site information directly on the Opportunity and Job rather than requiring a separate Property entity.</t>
+  </si>
+  <si>
+    <t>SA-002</t>
+  </si>
+  <si>
+    <t>FR-029</t>
+  </si>
+  <si>
+    <t>Opportunity and Job Site Information</t>
+  </si>
+  <si>
+    <t>The solution shall store site information directly on the Opportunity and copy the finalized site information to the Job when the work is awarded.</t>
+  </si>
+  <si>
+    <t>FR-030</t>
+  </si>
+  <si>
+    <t>Multiple Quotes per Opportunity</t>
+  </si>
+  <si>
+    <t>The solution shall support multiple quotes for one opportunity while requiring each quote to belong to exactly one opportunity.</t>
+  </si>
+  <si>
+    <t>FR-031</t>
+  </si>
+  <si>
+    <t>Bid-Budget Revisions</t>
+  </si>
+  <si>
+    <t>The solution shall support multiple bid-budget revisions for one quote and identify the current and final revisions.</t>
+  </si>
+  <si>
+    <t>FR-032</t>
+  </si>
+  <si>
+    <t>Accepted Quote-to-Job Lineage</t>
+  </si>
+  <si>
+    <t>The solution shall preserve accepted quote-to-job lineage through a Job Quote Source bridge and shall not implement an unresolved many-to-many relationship.</t>
+  </si>
+  <si>
+    <t>FR-033</t>
+  </si>
+  <si>
+    <t>Automatic Base Component</t>
+  </si>
+  <si>
+    <t>The solution shall automatically create a Base Contract component with suffix 000 when a Job is created.</t>
+  </si>
+  <si>
+    <t>FR-034</t>
+  </si>
+  <si>
+    <t>Job Component Types</t>
+  </si>
+  <si>
+    <t>The solution shall support Base Contract, Change Order, and Warranty Job Component types.</t>
+  </si>
+  <si>
+    <t>FR-035</t>
+  </si>
+  <si>
+    <t>Change-Order Component Numbering</t>
+  </si>
+  <si>
+    <t>The solution shall assign a sequential change-order component number when the change order is created and shall not reuse rejected or cancelled component numbers.</t>
+  </si>
+  <si>
+    <t>FR-036</t>
+  </si>
+  <si>
+    <t>Warranty Component Numbering</t>
+  </si>
+  <si>
+    <t>The solution shall assign warranty components a separate W01, W02, and subsequent numbering sequence.</t>
+  </si>
+  <si>
+    <t>FR-037</t>
+  </si>
+  <si>
+    <t>Component Type and Status</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Job Component Type and Job Component Status as separate attributes.</t>
+  </si>
+  <si>
+    <t>FR-038</t>
+  </si>
+  <si>
+    <t>Fixed Job Division</t>
+  </si>
+  <si>
+    <t>The solution shall assign each parent Job to exactly one division and shall retain that division throughout the full job lifecycle, including change orders and warranty work.</t>
+  </si>
+  <si>
+    <t>FR-039</t>
+  </si>
+  <si>
+    <t>Crew Independence</t>
+  </si>
+  <si>
+    <t>The solution shall maintain crews independently from divisions and shall allow employees to have one primary crew.</t>
+  </si>
+  <si>
+    <t>FR-040</t>
+  </si>
+  <si>
+    <t>Component Budget</t>
+  </si>
+  <si>
+    <t>The solution shall support no more than one Component Budget for each Job Component.</t>
+  </si>
+  <si>
+    <t>FR-041</t>
+  </si>
+  <si>
+    <t>Component Budget Detail</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Component Budget detail by Cost Code, Phase, and Cost Type.</t>
+  </si>
+  <si>
+    <t>FR-042</t>
+  </si>
+  <si>
+    <t>Component Budget Adjustments</t>
+  </si>
+  <si>
+    <t>The solution shall support budget adjustments at the component, cost-code, phase, and cost-type levels while associating each adjustment with exactly one Component Budget.</t>
+  </si>
+  <si>
+    <t>FR-043</t>
+  </si>
+  <si>
+    <t>Parent-Job Cost-Code Activation</t>
+  </si>
+  <si>
+    <t>The solution shall activate cost codes at the parent-job level, including new cost codes introduced through change orders.</t>
+  </si>
+  <si>
+    <t>FR-044</t>
+  </si>
+  <si>
+    <t>Standard Phase Activation</t>
+  </si>
+  <si>
+    <t>The solution shall activate Production phase 900 and Travel phase 905 for each active job cost code and shall activate Warranty phases 950 and 955 only when needed.</t>
+  </si>
+  <si>
+    <t>FR-045</t>
+  </si>
+  <si>
+    <t>Foreman Profitability Responsibility</t>
+  </si>
+  <si>
+    <t>The solution shall assign foreman profitability responsibility by Job and Cost Code and shall support shared responsibility percentages totaling 100 percent.</t>
+  </si>
+  <si>
+    <t>FR-046</t>
+  </si>
+  <si>
+    <t>Primary Crew Assignment</t>
+  </si>
+  <si>
+    <t>The solution shall maintain one current primary crew for each employee while allowing actual daily crew composition to differ.</t>
+  </si>
+  <si>
+    <t>FR-047</t>
+  </si>
+  <si>
+    <t>Daily Crew Derivation</t>
+  </si>
+  <si>
+    <t>The solution shall derive actual daily crew composition from employee time-entry activity rather than requiring a separate Daily Crew Assignment record.</t>
+  </si>
+  <si>
+    <t>FR-048</t>
+  </si>
+  <si>
+    <t>Time Entry Without Component</t>
+  </si>
+  <si>
+    <t>The solution shall capture employee time by employee, date, job, cost code, phase, labor code, start time, end time, and hours without requiring a Job Component.</t>
+  </si>
+  <si>
+    <t>FR-049</t>
+  </si>
+  <si>
+    <t>Estimated Daily Labor Cost</t>
+  </si>
+  <si>
+    <t>The solution shall calculate estimated daily labor cost using employee hours and the applicable estimated rate until final payroll cost is posted.</t>
+  </si>
+  <si>
+    <t>FR-050</t>
+  </si>
+  <si>
+    <t>Labor and Burden Separation</t>
+  </si>
+  <si>
+    <t>The solution shall calculate and report labor, tax burden, and indirect burden separately while preserving their relationship to the originating employee time entry.</t>
+  </si>
+  <si>
+    <t>FR-051</t>
+  </si>
+  <si>
+    <t>Equipment Usage Detail</t>
+  </si>
+  <si>
+    <t>The solution shall capture equipment usage by date, equipment unit, job, cost code, phase, and final approved usage hours.</t>
+  </si>
+  <si>
+    <t>FR-052</t>
+  </si>
+  <si>
+    <t>Effective-Dated Equipment Rates</t>
+  </si>
+  <si>
+    <t>The solution shall calculate estimated equipment cost using the effective-dated rate for the equipment unit and usage date.</t>
+  </si>
+  <si>
+    <t>FR-053</t>
+  </si>
+  <si>
+    <t>Material Transaction Detail</t>
+  </si>
+  <si>
+    <t>The solution shall capture material activity by date, job, cost code, phase, material item, quantity, unit of measure, applied unit cost, and source type.</t>
+  </si>
+  <si>
+    <t>FR-054</t>
+  </si>
+  <si>
+    <t>PO Line Ticket Fulfillment</t>
+  </si>
+  <si>
+    <t>The solution shall support one purchase-order line being fulfilled by one or many supplier-ticket lines.</t>
+  </si>
+  <si>
+    <t>FR-055</t>
+  </si>
+  <si>
+    <t>Supplier Ticket Matching</t>
+  </si>
+  <si>
+    <t>The solution shall associate each finalized supplier-ticket line with one applicable purchase-order line.</t>
+  </si>
+  <si>
+    <t>FR-056</t>
+  </si>
+  <si>
+    <t>Open Commitment Calculation</t>
+  </si>
+  <si>
+    <t>The solution shall calculate open commitment as the committed purchase-order amount less the invoiced amount.</t>
+  </si>
+  <si>
+    <t>FR-057</t>
+  </si>
+  <si>
+    <t>Posted Job-Cost Detail</t>
+  </si>
+  <si>
+    <t>The solution shall maintain posted job cost by posting date, work or usage date, job, cost code, phase, cost type, amount, quantity, source type, source record, and source-system transaction number.</t>
+  </si>
+  <si>
+    <t>FR-058</t>
+  </si>
+  <si>
+    <t>Estimated-to-Final Cost Replacement</t>
+  </si>
+  <si>
+    <t>The solution shall use estimated operational cost until final posted cost is available and shall replace the estimate with final cost without double-counting.</t>
+  </si>
+  <si>
+    <t>FR-059</t>
+  </si>
+  <si>
+    <t>Job-Cost Reversals</t>
+  </si>
+  <si>
+    <t>The solution shall correct posted job-cost errors through reversal and reposting while retaining the original transaction and correction lineage.</t>
+  </si>
+  <si>
+    <t>FR-060</t>
+  </si>
+  <si>
+    <t>Change-Order Actual Cost Treatment</t>
+  </si>
+  <si>
+    <t>The solution shall allow base and change-order actual labor, material, and equipment costs to remain combined at the parent Job and Cost Code level when separate field tracking is not practical.</t>
+  </si>
+  <si>
+    <t>FR-061</t>
+  </si>
+  <si>
+    <t>Warranty Cost Identification</t>
+  </si>
+  <si>
+    <t>The solution shall identify warranty actual costs using Warranty Production phase 950 and Warranty Travel phase 955.</t>
+  </si>
+  <si>
+    <t>FR-062</t>
+  </si>
+  <si>
+    <t>Customer Invoice Job Restriction</t>
+  </si>
+  <si>
+    <t>The solution shall allow each customer invoice to contain multiple line items but shall require the invoice to belong to exactly one Job.</t>
+  </si>
+  <si>
+    <t>FR-063</t>
+  </si>
+  <si>
+    <t>Total-Job Billing</t>
+  </si>
+  <si>
+    <t>The solution shall calculate billed revenue and billing analysis at the total parent-job level.</t>
+  </si>
+  <si>
+    <t>FR-064</t>
+  </si>
+  <si>
+    <t>Parent-Job WIP</t>
+  </si>
+  <si>
+    <t>The solution shall calculate WIP at the parent-job level.</t>
+  </si>
+  <si>
+    <t>FR-065</t>
+  </si>
+  <si>
+    <t>Approved Change Orders in WIP</t>
+  </si>
+  <si>
+    <t>The solution shall include only approved change-order revenue and budget in revised job revenue, revised budget, and WIP calculations.</t>
+  </si>
+  <si>
+    <t>FR-066</t>
+  </si>
+  <si>
+    <t>Warranty Treatment in WIP</t>
+  </si>
+  <si>
+    <t>The solution shall include warranty budget and warranty actual cost on the cost side of WIP while assigning zero revenue to warranty components.</t>
+  </si>
+  <si>
+    <t>FR-067</t>
+  </si>
+  <si>
+    <t>WIP Calculation Limits</t>
+  </si>
+  <si>
+    <t>The solution shall cap percent complete at 100 percent and earned revenue at revised job revenue.</t>
+  </si>
+  <si>
+    <t>FR-068</t>
+  </si>
+  <si>
+    <t>Current Job Forecast</t>
+  </si>
+  <si>
+    <t>The solution shall maintain one current forecast for each Job containing remaining cost to complete, forecast final cost, forecast final revenue, forecast final margin, notes, forecast date, and preparer.</t>
+  </si>
+  <si>
+    <t>FR-069</t>
+  </si>
+  <si>
+    <t>Forecast Detail</t>
+  </si>
+  <si>
+    <t>The solution shall support remaining-cost forecast detail by Cost Code with optional Cost Type detail.</t>
+  </si>
+  <si>
+    <t>FR-070</t>
+  </si>
+  <si>
+    <t>Forecast Replacement</t>
+  </si>
+  <si>
+    <t>The solution shall replace prior forecast values when a new current forecast is entered and shall not require formal historical forecast snapshots.</t>
+  </si>
+  <si>
+    <t>FR-071</t>
+  </si>
+  <si>
+    <t>Closed-Job Posting Restriction</t>
+  </si>
+  <si>
+    <t>The solution shall block operational and financial posting to a Job with a Closed status.</t>
+  </si>
+  <si>
+    <t>FR-072</t>
+  </si>
+  <si>
+    <t>Parent-Job Reopening</t>
+  </si>
+  <si>
+    <t>The solution shall require the parent Job to be formally reopened before processing late cost or warranty activity.</t>
+  </si>
+  <si>
+    <t>FR-073</t>
+  </si>
+  <si>
+    <t>Reopen and Reclose History</t>
+  </si>
+  <si>
+    <t>The solution shall retain Job reopen and reclose dates, reasons, users, and notes.</t>
+  </si>
+  <si>
+    <t>FR-074</t>
+  </si>
+  <si>
+    <t>Component Lifecycle Status</t>
+  </si>
+  <si>
+    <t>The solution shall maintain lifecycle status for each Job Component separately from the parent-job status.</t>
   </si>
 </sst>
 </file>
@@ -999,7 +1416,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1026,7 +1443,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2436,15 +2852,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{979FD651-F2D4-4BEE-84B1-39B645FFAE94}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="145.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="10"/>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="145.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2465,34 +2880,34 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>214</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="B2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D2" t="s">
+        <v>299</v>
+      </c>
+      <c r="E2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>24</v>
@@ -2500,16 +2915,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>223</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>24</v>
@@ -2517,16 +2932,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>226</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>24</v>
@@ -2534,16 +2949,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>229</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>24</v>
@@ -2551,16 +2966,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>232</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>24</v>
@@ -2568,16 +2983,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>235</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>24</v>
@@ -2585,16 +3000,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>238</v>
-      </c>
       <c r="D9" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>24</v>
@@ -2602,16 +3017,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>241</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>24</v>
@@ -2619,16 +3034,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>244</v>
-      </c>
       <c r="D11" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>24</v>
@@ -2636,16 +3051,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>247</v>
-      </c>
       <c r="D12" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>24</v>
@@ -2653,16 +3068,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>250</v>
-      </c>
       <c r="D13" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>24</v>
@@ -2670,16 +3085,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>253</v>
-      </c>
       <c r="D14" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>24</v>
@@ -2687,16 +3102,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>256</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>24</v>
@@ -2704,16 +3119,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="D16" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>24</v>
@@ -2721,16 +3136,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>262</v>
-      </c>
       <c r="D17" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>24</v>
@@ -2738,16 +3153,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="D18" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>24</v>
@@ -2755,16 +3170,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>268</v>
-      </c>
       <c r="D19" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>24</v>
@@ -2772,16 +3187,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>271</v>
-      </c>
       <c r="D20" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>24</v>
@@ -2789,16 +3204,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>274</v>
-      </c>
       <c r="D21" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>24</v>
@@ -2806,16 +3221,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>277</v>
-      </c>
       <c r="D22" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>24</v>
@@ -2823,16 +3238,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>280</v>
-      </c>
       <c r="D23" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>24</v>
@@ -2840,16 +3255,16 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>283</v>
-      </c>
       <c r="D24" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>24</v>
@@ -2857,16 +3272,16 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>286</v>
-      </c>
       <c r="D25" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>24</v>
@@ -2874,16 +3289,16 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>289</v>
-      </c>
       <c r="D26" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>24</v>
@@ -2891,16 +3306,16 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C27" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>292</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>24</v>
@@ -2908,16 +3323,16 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>295</v>
-      </c>
       <c r="D28" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>24</v>
@@ -2925,18 +3340,800 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>298</v>
-      </c>
       <c r="D29" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>300</v>
+      </c>
+      <c r="B30" t="s">
+        <v>301</v>
+      </c>
+      <c r="C30" t="s">
+        <v>302</v>
+      </c>
+      <c r="D30" t="s">
+        <v>299</v>
+      </c>
+      <c r="E30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>303</v>
+      </c>
+      <c r="B31" t="s">
+        <v>304</v>
+      </c>
+      <c r="C31" t="s">
+        <v>305</v>
+      </c>
+      <c r="D31" t="s">
+        <v>299</v>
+      </c>
+      <c r="E31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>306</v>
+      </c>
+      <c r="B32" t="s">
+        <v>307</v>
+      </c>
+      <c r="C32" t="s">
+        <v>308</v>
+      </c>
+      <c r="D32" t="s">
+        <v>299</v>
+      </c>
+      <c r="E32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>309</v>
+      </c>
+      <c r="B33" t="s">
+        <v>310</v>
+      </c>
+      <c r="C33" t="s">
+        <v>311</v>
+      </c>
+      <c r="D33" t="s">
+        <v>299</v>
+      </c>
+      <c r="E33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>312</v>
+      </c>
+      <c r="B34" t="s">
+        <v>313</v>
+      </c>
+      <c r="C34" t="s">
+        <v>314</v>
+      </c>
+      <c r="D34" t="s">
+        <v>299</v>
+      </c>
+      <c r="E34" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>315</v>
+      </c>
+      <c r="B35" t="s">
+        <v>316</v>
+      </c>
+      <c r="C35" t="s">
+        <v>317</v>
+      </c>
+      <c r="D35" t="s">
+        <v>299</v>
+      </c>
+      <c r="E35" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>318</v>
+      </c>
+      <c r="B36" t="s">
+        <v>319</v>
+      </c>
+      <c r="C36" t="s">
+        <v>320</v>
+      </c>
+      <c r="D36" t="s">
+        <v>299</v>
+      </c>
+      <c r="E36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>321</v>
+      </c>
+      <c r="B37" t="s">
+        <v>322</v>
+      </c>
+      <c r="C37" t="s">
+        <v>323</v>
+      </c>
+      <c r="D37" t="s">
+        <v>299</v>
+      </c>
+      <c r="E37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>324</v>
+      </c>
+      <c r="B38" t="s">
+        <v>325</v>
+      </c>
+      <c r="C38" t="s">
+        <v>326</v>
+      </c>
+      <c r="D38" t="s">
+        <v>299</v>
+      </c>
+      <c r="E38" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>327</v>
+      </c>
+      <c r="B39" t="s">
+        <v>328</v>
+      </c>
+      <c r="C39" t="s">
+        <v>329</v>
+      </c>
+      <c r="D39" t="s">
+        <v>299</v>
+      </c>
+      <c r="E39" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>330</v>
+      </c>
+      <c r="B40" t="s">
+        <v>331</v>
+      </c>
+      <c r="C40" t="s">
+        <v>332</v>
+      </c>
+      <c r="D40" t="s">
+        <v>299</v>
+      </c>
+      <c r="E40" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>333</v>
+      </c>
+      <c r="B41" t="s">
+        <v>334</v>
+      </c>
+      <c r="C41" t="s">
+        <v>335</v>
+      </c>
+      <c r="D41" t="s">
+        <v>299</v>
+      </c>
+      <c r="E41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>336</v>
+      </c>
+      <c r="B42" t="s">
+        <v>337</v>
+      </c>
+      <c r="C42" t="s">
+        <v>338</v>
+      </c>
+      <c r="D42" t="s">
+        <v>299</v>
+      </c>
+      <c r="E42" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>339</v>
+      </c>
+      <c r="B43" t="s">
+        <v>340</v>
+      </c>
+      <c r="C43" t="s">
+        <v>341</v>
+      </c>
+      <c r="D43" t="s">
+        <v>299</v>
+      </c>
+      <c r="E43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>342</v>
+      </c>
+      <c r="B44" t="s">
+        <v>343</v>
+      </c>
+      <c r="C44" t="s">
+        <v>344</v>
+      </c>
+      <c r="D44" t="s">
+        <v>299</v>
+      </c>
+      <c r="E44" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>345</v>
+      </c>
+      <c r="B45" t="s">
+        <v>346</v>
+      </c>
+      <c r="C45" t="s">
+        <v>347</v>
+      </c>
+      <c r="D45" t="s">
+        <v>299</v>
+      </c>
+      <c r="E45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" t="s">
+        <v>349</v>
+      </c>
+      <c r="C46" t="s">
+        <v>350</v>
+      </c>
+      <c r="D46" t="s">
+        <v>299</v>
+      </c>
+      <c r="E46" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>351</v>
+      </c>
+      <c r="B47" t="s">
+        <v>352</v>
+      </c>
+      <c r="C47" t="s">
+        <v>353</v>
+      </c>
+      <c r="D47" t="s">
+        <v>299</v>
+      </c>
+      <c r="E47" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>354</v>
+      </c>
+      <c r="B48" t="s">
+        <v>355</v>
+      </c>
+      <c r="C48" t="s">
+        <v>356</v>
+      </c>
+      <c r="D48" t="s">
+        <v>299</v>
+      </c>
+      <c r="E48" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>357</v>
+      </c>
+      <c r="B49" t="s">
+        <v>358</v>
+      </c>
+      <c r="C49" t="s">
+        <v>359</v>
+      </c>
+      <c r="D49" t="s">
+        <v>299</v>
+      </c>
+      <c r="E49" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>360</v>
+      </c>
+      <c r="B50" t="s">
+        <v>361</v>
+      </c>
+      <c r="C50" t="s">
+        <v>362</v>
+      </c>
+      <c r="D50" t="s">
+        <v>299</v>
+      </c>
+      <c r="E50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>363</v>
+      </c>
+      <c r="B51" t="s">
+        <v>364</v>
+      </c>
+      <c r="C51" t="s">
+        <v>365</v>
+      </c>
+      <c r="D51" t="s">
+        <v>299</v>
+      </c>
+      <c r="E51" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>366</v>
+      </c>
+      <c r="B52" t="s">
+        <v>367</v>
+      </c>
+      <c r="C52" t="s">
+        <v>368</v>
+      </c>
+      <c r="D52" t="s">
+        <v>299</v>
+      </c>
+      <c r="E52" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>369</v>
+      </c>
+      <c r="B53" t="s">
+        <v>370</v>
+      </c>
+      <c r="C53" t="s">
+        <v>371</v>
+      </c>
+      <c r="D53" t="s">
+        <v>299</v>
+      </c>
+      <c r="E53" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>372</v>
+      </c>
+      <c r="B54" t="s">
+        <v>373</v>
+      </c>
+      <c r="C54" t="s">
+        <v>374</v>
+      </c>
+      <c r="D54" t="s">
+        <v>299</v>
+      </c>
+      <c r="E54" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>375</v>
+      </c>
+      <c r="B55" t="s">
+        <v>376</v>
+      </c>
+      <c r="C55" t="s">
+        <v>377</v>
+      </c>
+      <c r="D55" t="s">
+        <v>299</v>
+      </c>
+      <c r="E55" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>378</v>
+      </c>
+      <c r="B56" t="s">
+        <v>379</v>
+      </c>
+      <c r="C56" t="s">
+        <v>380</v>
+      </c>
+      <c r="D56" t="s">
+        <v>299</v>
+      </c>
+      <c r="E56" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>381</v>
+      </c>
+      <c r="B57" t="s">
+        <v>382</v>
+      </c>
+      <c r="C57" t="s">
+        <v>383</v>
+      </c>
+      <c r="D57" t="s">
+        <v>299</v>
+      </c>
+      <c r="E57" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>384</v>
+      </c>
+      <c r="B58" t="s">
+        <v>385</v>
+      </c>
+      <c r="C58" t="s">
+        <v>386</v>
+      </c>
+      <c r="D58" t="s">
+        <v>299</v>
+      </c>
+      <c r="E58" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>387</v>
+      </c>
+      <c r="B59" t="s">
+        <v>388</v>
+      </c>
+      <c r="C59" t="s">
+        <v>389</v>
+      </c>
+      <c r="D59" t="s">
+        <v>299</v>
+      </c>
+      <c r="E59" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>390</v>
+      </c>
+      <c r="B60" t="s">
+        <v>391</v>
+      </c>
+      <c r="C60" t="s">
+        <v>392</v>
+      </c>
+      <c r="D60" t="s">
+        <v>299</v>
+      </c>
+      <c r="E60" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>393</v>
+      </c>
+      <c r="B61" t="s">
+        <v>394</v>
+      </c>
+      <c r="C61" t="s">
+        <v>395</v>
+      </c>
+      <c r="D61" t="s">
+        <v>299</v>
+      </c>
+      <c r="E61" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>396</v>
+      </c>
+      <c r="B62" t="s">
+        <v>397</v>
+      </c>
+      <c r="C62" t="s">
+        <v>398</v>
+      </c>
+      <c r="D62" t="s">
+        <v>299</v>
+      </c>
+      <c r="E62" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>399</v>
+      </c>
+      <c r="B63" t="s">
+        <v>400</v>
+      </c>
+      <c r="C63" t="s">
+        <v>401</v>
+      </c>
+      <c r="D63" t="s">
+        <v>299</v>
+      </c>
+      <c r="E63" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>402</v>
+      </c>
+      <c r="B64" t="s">
+        <v>403</v>
+      </c>
+      <c r="C64" t="s">
+        <v>404</v>
+      </c>
+      <c r="D64" t="s">
+        <v>299</v>
+      </c>
+      <c r="E64" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>405</v>
+      </c>
+      <c r="B65" t="s">
+        <v>406</v>
+      </c>
+      <c r="C65" t="s">
+        <v>407</v>
+      </c>
+      <c r="D65" t="s">
+        <v>299</v>
+      </c>
+      <c r="E65" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>408</v>
+      </c>
+      <c r="B66" t="s">
+        <v>409</v>
+      </c>
+      <c r="C66" t="s">
+        <v>410</v>
+      </c>
+      <c r="D66" t="s">
+        <v>299</v>
+      </c>
+      <c r="E66" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>411</v>
+      </c>
+      <c r="B67" t="s">
+        <v>412</v>
+      </c>
+      <c r="C67" t="s">
+        <v>413</v>
+      </c>
+      <c r="D67" t="s">
+        <v>299</v>
+      </c>
+      <c r="E67" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>414</v>
+      </c>
+      <c r="B68" t="s">
+        <v>415</v>
+      </c>
+      <c r="C68" t="s">
+        <v>416</v>
+      </c>
+      <c r="D68" t="s">
+        <v>299</v>
+      </c>
+      <c r="E68" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>417</v>
+      </c>
+      <c r="B69" t="s">
+        <v>418</v>
+      </c>
+      <c r="C69" t="s">
+        <v>419</v>
+      </c>
+      <c r="D69" t="s">
+        <v>299</v>
+      </c>
+      <c r="E69" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>420</v>
+      </c>
+      <c r="B70" t="s">
+        <v>421</v>
+      </c>
+      <c r="C70" t="s">
+        <v>422</v>
+      </c>
+      <c r="D70" t="s">
+        <v>299</v>
+      </c>
+      <c r="E70" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>423</v>
+      </c>
+      <c r="B71" t="s">
+        <v>424</v>
+      </c>
+      <c r="C71" t="s">
+        <v>425</v>
+      </c>
+      <c r="D71" t="s">
+        <v>299</v>
+      </c>
+      <c r="E71" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>426</v>
+      </c>
+      <c r="B72" t="s">
+        <v>427</v>
+      </c>
+      <c r="C72" t="s">
+        <v>428</v>
+      </c>
+      <c r="D72" t="s">
+        <v>299</v>
+      </c>
+      <c r="E72" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>429</v>
+      </c>
+      <c r="B73" t="s">
+        <v>430</v>
+      </c>
+      <c r="C73" t="s">
+        <v>431</v>
+      </c>
+      <c r="D73" t="s">
+        <v>299</v>
+      </c>
+      <c r="E73" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>432</v>
+      </c>
+      <c r="B74" t="s">
+        <v>433</v>
+      </c>
+      <c r="C74" t="s">
+        <v>434</v>
+      </c>
+      <c r="D74" t="s">
+        <v>299</v>
+      </c>
+      <c r="E74" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>435</v>
+      </c>
+      <c r="B75" t="s">
+        <v>436</v>
+      </c>
+      <c r="C75" t="s">
+        <v>437</v>
+      </c>
+      <c r="D75" t="s">
+        <v>299</v>
+      </c>
+      <c r="E75" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Sa-003 logical data model
</commit_message>
<xml_diff>
--- a/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
+++ b/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd01d60e8fdc72b3/Projects/Construction_Analytics_Platform/Documentation/Formal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="139" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9FAD9689-C9EA-4C39-AF0C-C98BC151269C}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{913AA438-1A64-45F0-9FD5-12D0AFEF00BA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" activeTab="2" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="630">
   <si>
     <t>KPI</t>
   </si>
@@ -1358,6 +1358,582 @@
   </si>
   <si>
     <t>The solution shall maintain lifecycle status for each Job Component separately from the parent-job status.</t>
+  </si>
+  <si>
+    <t>FR-075</t>
+  </si>
+  <si>
+    <t>Logical Subject Areas</t>
+  </si>
+  <si>
+    <t>The solution shall organize the logical data model into Customer and Sales, Estimating and Bid Budget, Job and Scope, Budget and Cost Structure, Workforce and Responsibility, Field Activity, Equipment, Materials and Inventory, Purchasing and Commitments, Posted Job Cost, Billing and Revenue, WIP and Forecasting, and Reference and Shared Master Data subject areas.</t>
+  </si>
+  <si>
+    <t>SA-003</t>
+  </si>
+  <si>
+    <t>FR-076</t>
+  </si>
+  <si>
+    <t>Subject-Area Ownership</t>
+  </si>
+  <si>
+    <t>The solution shall assign each logical entity to one primary subject-area owner while documenting all cross-subject relationships.</t>
+  </si>
+  <si>
+    <t>FR-077</t>
+  </si>
+  <si>
+    <t>Sales and Estimating Separation</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Customer, Opportunity, and Quote within Customer and Sales while maintaining Bid Budget Revision and related estimating detail within Estimating and Bid Budget.</t>
+  </si>
+  <si>
+    <t>FR-078</t>
+  </si>
+  <si>
+    <t>Quote Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat Quote as the authoritative customer-facing proposal before job award.</t>
+  </si>
+  <si>
+    <t>FR-079</t>
+  </si>
+  <si>
+    <t>Bid Budget Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat the final Bid Budget Revision as the authoritative internal estimate supporting the submitted Quote.</t>
+  </si>
+  <si>
+    <t>FR-080</t>
+  </si>
+  <si>
+    <t>Job Post-Award Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat Job as the authoritative record for the awarded work after job creation.</t>
+  </si>
+  <si>
+    <t>FR-081</t>
+  </si>
+  <si>
+    <t>Original Quote Budget Retention</t>
+  </si>
+  <si>
+    <t>The solution shall retain original Quote Budgets unchanged as historical estimating records.</t>
+  </si>
+  <si>
+    <t>FR-082</t>
+  </si>
+  <si>
+    <t>New Final Job Budget</t>
+  </si>
+  <si>
+    <t>The solution shall create a new final Job Budget for awarded work rather than mathematically combining the budgets of accepted Quotes.</t>
+  </si>
+  <si>
+    <t>FR-083</t>
+  </si>
+  <si>
+    <t>Job Component Ownership</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Job Component within the Job and Scope subject area.</t>
+  </si>
+  <si>
+    <t>FR-084</t>
+  </si>
+  <si>
+    <t>Component Budget Ownership</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Component Budget within the Budget and Cost Structure subject area.</t>
+  </si>
+  <si>
+    <t>FR-085</t>
+  </si>
+  <si>
+    <t>Current Job Roles</t>
+  </si>
+  <si>
+    <t>The solution shall store the current Project Manager, Superintendent, Sales Representative, Estimator, and Coordinator directly on the Job.</t>
+  </si>
+  <si>
+    <t>FR-086</t>
+  </si>
+  <si>
+    <t>Job Role History</t>
+  </si>
+  <si>
+    <t>The initial solution shall not require historical tracking of Job role assignments.</t>
+  </si>
+  <si>
+    <t>FR-087</t>
+  </si>
+  <si>
+    <t>Responsible Foreman</t>
+  </si>
+  <si>
+    <t>The solution shall assign Responsible Foreman by Job and Cost Code for incentive, profitability, fade/gain, and long-term performance analysis.</t>
+  </si>
+  <si>
+    <t>FR-088</t>
+  </si>
+  <si>
+    <t>Daily Foreman</t>
+  </si>
+  <si>
+    <t>The solution shall separately identify the Daily Foreman who actually supervised work on a specific date and task.</t>
+  </si>
+  <si>
+    <t>FR-089</t>
+  </si>
+  <si>
+    <t>Multiple Foremen per Job Day</t>
+  </si>
+  <si>
+    <t>The solution shall support multiple foremen supervising different tasks on the same Job during the same date and time period.</t>
+  </si>
+  <si>
+    <t>FR-090</t>
+  </si>
+  <si>
+    <t>Employee Foreman Changes</t>
+  </si>
+  <si>
+    <t>The solution shall support an Employee working under more than one Daily Foreman during the same day.</t>
+  </si>
+  <si>
+    <t>FR-091</t>
+  </si>
+  <si>
+    <t>Employee Labor Segments</t>
+  </si>
+  <si>
+    <t>The solution shall preserve separate labor segments when an Employee changes Foreman, Cost Code, Phase, or task during the day.</t>
+  </si>
+  <si>
+    <t>FR-092</t>
+  </si>
+  <si>
+    <t>Derived Daily Work Groups</t>
+  </si>
+  <si>
+    <t>The solution shall derive Daily Work Groups from imported labor records using Job, Work Date, and Foreman.</t>
+  </si>
+  <si>
+    <t>FR-093</t>
+  </si>
+  <si>
+    <t>Multiple Cost Codes per Work Group</t>
+  </si>
+  <si>
+    <t>The solution shall allow one Daily Work Group to perform work under multiple Cost Codes on the same Job and date.</t>
+  </si>
+  <si>
+    <t>FR-094</t>
+  </si>
+  <si>
+    <t>Daily Work Assignment</t>
+  </si>
+  <si>
+    <t>The solution shall represent task-level supervision within a Daily Work Group through Daily Work Assignment records or derived structures.</t>
+  </si>
+  <si>
+    <t>FR-095</t>
+  </si>
+  <si>
+    <t>Daily Production Ownership</t>
+  </si>
+  <si>
+    <t>The solution shall associate Daily Production with Work Date, Job, Daily Foreman, Cost Code, and Production Measure.</t>
+  </si>
+  <si>
+    <t>FR-096</t>
+  </si>
+  <si>
+    <t>Multiple Production Measures</t>
+  </si>
+  <si>
+    <t>The solution shall allow multiple production measures for the same Job, Daily Foreman, Cost Code, and Work Date.</t>
+  </si>
+  <si>
+    <t>FR-097</t>
+  </si>
+  <si>
+    <t>Equipment Usage Ownership</t>
+  </si>
+  <si>
+    <t>The solution shall maintain Equipment Usage within Field Activity while maintaining Equipment Unit, Equipment Rate History, Equipment Type, and Equipment Status within Equipment.</t>
+  </si>
+  <si>
+    <t>FR-098</t>
+  </si>
+  <si>
+    <t>Operational Delay Hours</t>
+  </si>
+  <si>
+    <t>The solution shall store entered delay hours without requiring exact delay start and end times.</t>
+  </si>
+  <si>
+    <t>FR-099</t>
+  </si>
+  <si>
+    <t>Operational Delay Scope</t>
+  </si>
+  <si>
+    <t>The solution shall allow an Operational Delay to reference a Daily Work Group, Daily Work Assignment, Cost Code, Equipment Unit, Employee, or a combination of these.</t>
+  </si>
+  <si>
+    <t>FR-100</t>
+  </si>
+  <si>
+    <t>Delay Scope Identification</t>
+  </si>
+  <si>
+    <t>The solution shall identify the scope of each Operational Delay so delay hours are not overstated across affected resources.</t>
+  </si>
+  <si>
+    <t>FR-101</t>
+  </si>
+  <si>
+    <t>Imported Source Records</t>
+  </si>
+  <si>
+    <t>The solution shall import operational and financial records from external source systems rather than requiring direct entry into the analytics solution.</t>
+  </si>
+  <si>
+    <t>FR-102</t>
+  </si>
+  <si>
+    <t>Source-System Lineage</t>
+  </si>
+  <si>
+    <t>The solution shall retain source system, source record identifier, source-created date, source-modified date, first-imported date, last-imported date, import batch, and record version where available.</t>
+  </si>
+  <si>
+    <t>FR-103</t>
+  </si>
+  <si>
+    <t>Operational Record Corrections</t>
+  </si>
+  <si>
+    <t>The solution shall update an existing imported operational record when a corrected source record is received while retaining audit information.</t>
+  </si>
+  <si>
+    <t>FR-104</t>
+  </si>
+  <si>
+    <t>Posted Financial Corrections</t>
+  </si>
+  <si>
+    <t>The solution shall preserve source-system reversal and reposting transactions for posted financial corrections.</t>
+  </si>
+  <si>
+    <t>FR-105</t>
+  </si>
+  <si>
+    <t>Operational Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat operational records as authoritative for activity hours, quantities, assignments, and production.</t>
+  </si>
+  <si>
+    <t>FR-106</t>
+  </si>
+  <si>
+    <t>Posted Cost Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat Posted Job Cost as authoritative for final financial cost.</t>
+  </si>
+  <si>
+    <t>FR-107</t>
+  </si>
+  <si>
+    <t>Direct Cost Matching</t>
+  </si>
+  <si>
+    <t>The solution shall use direct source-record identifiers to match operational records to Posted Job Cost whenever available.</t>
+  </si>
+  <si>
+    <t>FR-108</t>
+  </si>
+  <si>
+    <t>Rule-Based Cost Matching</t>
+  </si>
+  <si>
+    <t>The solution shall support controlled rule-based matching when direct source linkage is unavailable.</t>
+  </si>
+  <si>
+    <t>FR-109</t>
+  </si>
+  <si>
+    <t>Cost Matching Criteria</t>
+  </si>
+  <si>
+    <t>Rule-based matching may use Job, date, Cost Code, Phase, Cost Type, source type, quantity, hours, Employee, Equipment Unit, Material Item, Vendor, source batch, or transaction number.</t>
+  </si>
+  <si>
+    <t>FR-110</t>
+  </si>
+  <si>
+    <t>Matching Status</t>
+  </si>
+  <si>
+    <t>The solution shall support Direct Match, Rule-Based Match, Ambiguous Match, Unmatched, and Not Applicable matching statuses.</t>
+  </si>
+  <si>
+    <t>FR-111</t>
+  </si>
+  <si>
+    <t>Estimated Cost Replacement</t>
+  </si>
+  <si>
+    <t>The solution shall remove estimated operational cost from financial reporting only after a corresponding final Posted Job Cost is matched with sufficient confidence.</t>
+  </si>
+  <si>
+    <t>FR-112</t>
+  </si>
+  <si>
+    <t>Supplier Ticket Independence</t>
+  </si>
+  <si>
+    <t>The solution shall import Supplier Ticket Lines independently from Material Transactions.</t>
+  </si>
+  <si>
+    <t>FR-113</t>
+  </si>
+  <si>
+    <t>Material Transaction Independence</t>
+  </si>
+  <si>
+    <t>The solution shall not automatically create a Material Transaction from a Supplier Ticket Line within the analytics solution.</t>
+  </si>
+  <si>
+    <t>FR-114</t>
+  </si>
+  <si>
+    <t>Supplier Material Reconciliation</t>
+  </si>
+  <si>
+    <t>The solution shall support reconciliation between Supplier Ticket Lines and Material Transactions, including one-to-many and many-to-one relationships where necessary.</t>
+  </si>
+  <si>
+    <t>FR-115</t>
+  </si>
+  <si>
+    <t>Delivered Quantity Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat Supplier Ticket Line as authoritative for delivered quantity.</t>
+  </si>
+  <si>
+    <t>FR-116</t>
+  </si>
+  <si>
+    <t>Invoiced Quantity and Cost Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat Supplier Invoice Line as authoritative for invoiced quantity and cost.</t>
+  </si>
+  <si>
+    <t>FR-117</t>
+  </si>
+  <si>
+    <t>Material Quantity and Applied Cost Authority</t>
+  </si>
+  <si>
+    <t>The solution shall treat Material Transaction as authoritative for job-level material quantity and applied cost.</t>
+  </si>
+  <si>
+    <t>FR-118</t>
+  </si>
+  <si>
+    <t>Billing and WIP Separation</t>
+  </si>
+  <si>
+    <t>The solution shall maintain customer billing transactions separately from WIP, forecasting, earned revenue, over/under billing, and profitability calculations.</t>
+  </si>
+  <si>
+    <t>FR-119</t>
+  </si>
+  <si>
+    <t>Dynamic Current WIP</t>
+  </si>
+  <si>
+    <t>The solution shall calculate current WIP dynamically from current budget, cost, commitment, billing, and forecast data.</t>
+  </si>
+  <si>
+    <t>FR-120</t>
+  </si>
+  <si>
+    <t>Weekly WIP Snapshots</t>
+  </si>
+  <si>
+    <t>The solution shall create and retain weekly WIP snapshots for operational reporting.</t>
+  </si>
+  <si>
+    <t>FR-121</t>
+  </si>
+  <si>
+    <t>Month-End WIP Snapshots</t>
+  </si>
+  <si>
+    <t>The solution shall create and retain month-end WIP snapshots for financial reporting.</t>
+  </si>
+  <si>
+    <t>FR-122</t>
+  </si>
+  <si>
+    <t>WIP Snapshot Grain</t>
+  </si>
+  <si>
+    <t>The solution shall store WIP Snapshots at the Job and Reporting Date grain.</t>
+  </si>
+  <si>
+    <t>FR-123</t>
+  </si>
+  <si>
+    <t>Snapshot Classification</t>
+  </si>
+  <si>
+    <t>The solution shall identify each WIP Snapshot as Weekly, Month-End, or both.</t>
+  </si>
+  <si>
+    <t>FR-124</t>
+  </si>
+  <si>
+    <t>WIP Snapshot Retention</t>
+  </si>
+  <si>
+    <t>The solution shall retain prior WIP Snapshots without overwriting them.</t>
+  </si>
+  <si>
+    <t>FR-125</t>
+  </si>
+  <si>
+    <t>WIP Period Deltas</t>
+  </si>
+  <si>
+    <t>The solution shall support week-to-week and month-to-month change analysis by comparing consecutive WIP Snapshots.</t>
+  </si>
+  <si>
+    <t>FR-126</t>
+  </si>
+  <si>
+    <t>Current Forecast</t>
+  </si>
+  <si>
+    <t>The solution shall maintain one current editable forecast per Job.</t>
+  </si>
+  <si>
+    <t>FR-127</t>
+  </si>
+  <si>
+    <t>Forecast Snapshot History</t>
+  </si>
+  <si>
+    <t>The solution shall preserve the forecast values used at each reporting cutoff within the related WIP Snapshot.</t>
+  </si>
+  <si>
+    <t>FR-128</t>
+  </si>
+  <si>
+    <t>Global WIP Week-End Day</t>
+  </si>
+  <si>
+    <t>The solution shall use a globally configured fixed day of the week for weekly WIP reporting.</t>
+  </si>
+  <si>
+    <t>FR-129</t>
+  </si>
+  <si>
+    <t>WIP Week-End Permanence</t>
+  </si>
+  <si>
+    <t>The configured WIP week-ending day shall apply to all Jobs and shall not change after implementation without a formal conversion process.</t>
+  </si>
+  <si>
+    <t>FR-130</t>
+  </si>
+  <si>
+    <t>Effective-Dated Labor Rates</t>
+  </si>
+  <si>
+    <t>The solution shall retain effective-dated Employee labor-rate history.</t>
+  </si>
+  <si>
+    <t>FR-131</t>
+  </si>
+  <si>
+    <t>The solution shall retain effective-dated Equipment-rate history.</t>
+  </si>
+  <si>
+    <t>FR-132</t>
+  </si>
+  <si>
+    <t>Effective-Dated Material Costs</t>
+  </si>
+  <si>
+    <t>The solution shall retain effective-dated Material standard-cost history.</t>
+  </si>
+  <si>
+    <t>FR-133</t>
+  </si>
+  <si>
+    <t>Effective-Dated Crew Assignments</t>
+  </si>
+  <si>
+    <t>The solution shall retain effective-dated Employee primary-crew assignment history.</t>
+  </si>
+  <si>
+    <t>FR-134</t>
+  </si>
+  <si>
+    <t>Effective-Date Overlap</t>
+  </si>
+  <si>
+    <t>The solution shall prohibit overlapping effective-date ranges for the same entity and rate, cost, or assignment type.</t>
+  </si>
+  <si>
+    <t>FR-135</t>
+  </si>
+  <si>
+    <t>Historical Applied Rates</t>
+  </si>
+  <si>
+    <t>The solution shall retain applied rates and costs on transactions and shall not recalculate historical transactions when master rates or costs change.</t>
+  </si>
+  <si>
+    <t>FR-136</t>
+  </si>
+  <si>
+    <t>Global Configuration</t>
+  </si>
+  <si>
+    <t>The solution shall provide a Global Configuration entity for company-wide reporting and processing settings.</t>
+  </si>
+  <si>
+    <t>FR-137</t>
+  </si>
+  <si>
+    <t>Global Configuration Values</t>
+  </si>
+  <si>
+    <t>Global Configuration shall support WIP week-ending day, fiscal year-end, standard workweek, snapshot requirements, variance tolerances, closed-job posting rules, default phases, reporting currency, reporting time zone, and WIP or forecast calculation options.</t>
+  </si>
+  <si>
+    <t>FR-138</t>
+  </si>
+  <si>
+    <t>Configuration Change Control</t>
+  </si>
+  <si>
+    <t>The solution shall lock configuration values that affect historical comparability after implementation or require a controlled conversion process before changing them.</t>
   </si>
 </sst>
 </file>
@@ -2852,7 +3428,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{979FD651-F2D4-4BEE-84B1-39B645FFAE94}">
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
@@ -4134,6 +4710,1094 @@
         <v>299</v>
       </c>
       <c r="E75" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>438</v>
+      </c>
+      <c r="B76" t="s">
+        <v>439</v>
+      </c>
+      <c r="C76" t="s">
+        <v>440</v>
+      </c>
+      <c r="D76" t="s">
+        <v>441</v>
+      </c>
+      <c r="E76" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>442</v>
+      </c>
+      <c r="B77" t="s">
+        <v>443</v>
+      </c>
+      <c r="C77" t="s">
+        <v>444</v>
+      </c>
+      <c r="D77" t="s">
+        <v>441</v>
+      </c>
+      <c r="E77" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>445</v>
+      </c>
+      <c r="B78" t="s">
+        <v>446</v>
+      </c>
+      <c r="C78" t="s">
+        <v>447</v>
+      </c>
+      <c r="D78" t="s">
+        <v>441</v>
+      </c>
+      <c r="E78" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>448</v>
+      </c>
+      <c r="B79" t="s">
+        <v>449</v>
+      </c>
+      <c r="C79" t="s">
+        <v>450</v>
+      </c>
+      <c r="D79" t="s">
+        <v>441</v>
+      </c>
+      <c r="E79" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>451</v>
+      </c>
+      <c r="B80" t="s">
+        <v>452</v>
+      </c>
+      <c r="C80" t="s">
+        <v>453</v>
+      </c>
+      <c r="D80" t="s">
+        <v>441</v>
+      </c>
+      <c r="E80" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>454</v>
+      </c>
+      <c r="B81" t="s">
+        <v>455</v>
+      </c>
+      <c r="C81" t="s">
+        <v>456</v>
+      </c>
+      <c r="D81" t="s">
+        <v>441</v>
+      </c>
+      <c r="E81" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>457</v>
+      </c>
+      <c r="B82" t="s">
+        <v>458</v>
+      </c>
+      <c r="C82" t="s">
+        <v>459</v>
+      </c>
+      <c r="D82" t="s">
+        <v>441</v>
+      </c>
+      <c r="E82" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>460</v>
+      </c>
+      <c r="B83" t="s">
+        <v>461</v>
+      </c>
+      <c r="C83" t="s">
+        <v>462</v>
+      </c>
+      <c r="D83" t="s">
+        <v>441</v>
+      </c>
+      <c r="E83" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>463</v>
+      </c>
+      <c r="B84" t="s">
+        <v>464</v>
+      </c>
+      <c r="C84" t="s">
+        <v>465</v>
+      </c>
+      <c r="D84" t="s">
+        <v>441</v>
+      </c>
+      <c r="E84" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>466</v>
+      </c>
+      <c r="B85" t="s">
+        <v>467</v>
+      </c>
+      <c r="C85" t="s">
+        <v>468</v>
+      </c>
+      <c r="D85" t="s">
+        <v>441</v>
+      </c>
+      <c r="E85" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>469</v>
+      </c>
+      <c r="B86" t="s">
+        <v>470</v>
+      </c>
+      <c r="C86" t="s">
+        <v>471</v>
+      </c>
+      <c r="D86" t="s">
+        <v>441</v>
+      </c>
+      <c r="E86" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>472</v>
+      </c>
+      <c r="B87" t="s">
+        <v>473</v>
+      </c>
+      <c r="C87" t="s">
+        <v>474</v>
+      </c>
+      <c r="D87" t="s">
+        <v>441</v>
+      </c>
+      <c r="E87" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>475</v>
+      </c>
+      <c r="B88" t="s">
+        <v>476</v>
+      </c>
+      <c r="C88" t="s">
+        <v>477</v>
+      </c>
+      <c r="D88" t="s">
+        <v>441</v>
+      </c>
+      <c r="E88" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>478</v>
+      </c>
+      <c r="B89" t="s">
+        <v>479</v>
+      </c>
+      <c r="C89" t="s">
+        <v>480</v>
+      </c>
+      <c r="D89" t="s">
+        <v>441</v>
+      </c>
+      <c r="E89" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>481</v>
+      </c>
+      <c r="B90" t="s">
+        <v>482</v>
+      </c>
+      <c r="C90" t="s">
+        <v>483</v>
+      </c>
+      <c r="D90" t="s">
+        <v>441</v>
+      </c>
+      <c r="E90" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>484</v>
+      </c>
+      <c r="B91" t="s">
+        <v>485</v>
+      </c>
+      <c r="C91" t="s">
+        <v>486</v>
+      </c>
+      <c r="D91" t="s">
+        <v>441</v>
+      </c>
+      <c r="E91" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>487</v>
+      </c>
+      <c r="B92" t="s">
+        <v>488</v>
+      </c>
+      <c r="C92" t="s">
+        <v>489</v>
+      </c>
+      <c r="D92" t="s">
+        <v>441</v>
+      </c>
+      <c r="E92" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>490</v>
+      </c>
+      <c r="B93" t="s">
+        <v>491</v>
+      </c>
+      <c r="C93" t="s">
+        <v>492</v>
+      </c>
+      <c r="D93" t="s">
+        <v>441</v>
+      </c>
+      <c r="E93" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>493</v>
+      </c>
+      <c r="B94" t="s">
+        <v>494</v>
+      </c>
+      <c r="C94" t="s">
+        <v>495</v>
+      </c>
+      <c r="D94" t="s">
+        <v>441</v>
+      </c>
+      <c r="E94" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>496</v>
+      </c>
+      <c r="B95" t="s">
+        <v>497</v>
+      </c>
+      <c r="C95" t="s">
+        <v>498</v>
+      </c>
+      <c r="D95" t="s">
+        <v>441</v>
+      </c>
+      <c r="E95" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>499</v>
+      </c>
+      <c r="B96" t="s">
+        <v>500</v>
+      </c>
+      <c r="C96" t="s">
+        <v>501</v>
+      </c>
+      <c r="D96" t="s">
+        <v>441</v>
+      </c>
+      <c r="E96" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>502</v>
+      </c>
+      <c r="B97" t="s">
+        <v>503</v>
+      </c>
+      <c r="C97" t="s">
+        <v>504</v>
+      </c>
+      <c r="D97" t="s">
+        <v>441</v>
+      </c>
+      <c r="E97" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>505</v>
+      </c>
+      <c r="B98" t="s">
+        <v>506</v>
+      </c>
+      <c r="C98" t="s">
+        <v>507</v>
+      </c>
+      <c r="D98" t="s">
+        <v>441</v>
+      </c>
+      <c r="E98" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>508</v>
+      </c>
+      <c r="B99" t="s">
+        <v>509</v>
+      </c>
+      <c r="C99" t="s">
+        <v>510</v>
+      </c>
+      <c r="D99" t="s">
+        <v>441</v>
+      </c>
+      <c r="E99" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>511</v>
+      </c>
+      <c r="B100" t="s">
+        <v>512</v>
+      </c>
+      <c r="C100" t="s">
+        <v>513</v>
+      </c>
+      <c r="D100" t="s">
+        <v>441</v>
+      </c>
+      <c r="E100" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>514</v>
+      </c>
+      <c r="B101" t="s">
+        <v>515</v>
+      </c>
+      <c r="C101" t="s">
+        <v>516</v>
+      </c>
+      <c r="D101" t="s">
+        <v>441</v>
+      </c>
+      <c r="E101" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>517</v>
+      </c>
+      <c r="B102" t="s">
+        <v>518</v>
+      </c>
+      <c r="C102" t="s">
+        <v>519</v>
+      </c>
+      <c r="D102" t="s">
+        <v>441</v>
+      </c>
+      <c r="E102" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>520</v>
+      </c>
+      <c r="B103" t="s">
+        <v>521</v>
+      </c>
+      <c r="C103" t="s">
+        <v>522</v>
+      </c>
+      <c r="D103" t="s">
+        <v>441</v>
+      </c>
+      <c r="E103" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>523</v>
+      </c>
+      <c r="B104" t="s">
+        <v>524</v>
+      </c>
+      <c r="C104" t="s">
+        <v>525</v>
+      </c>
+      <c r="D104" t="s">
+        <v>441</v>
+      </c>
+      <c r="E104" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>526</v>
+      </c>
+      <c r="B105" t="s">
+        <v>527</v>
+      </c>
+      <c r="C105" t="s">
+        <v>528</v>
+      </c>
+      <c r="D105" t="s">
+        <v>441</v>
+      </c>
+      <c r="E105" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>529</v>
+      </c>
+      <c r="B106" t="s">
+        <v>530</v>
+      </c>
+      <c r="C106" t="s">
+        <v>531</v>
+      </c>
+      <c r="D106" t="s">
+        <v>441</v>
+      </c>
+      <c r="E106" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>532</v>
+      </c>
+      <c r="B107" t="s">
+        <v>533</v>
+      </c>
+      <c r="C107" t="s">
+        <v>534</v>
+      </c>
+      <c r="D107" t="s">
+        <v>441</v>
+      </c>
+      <c r="E107" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>535</v>
+      </c>
+      <c r="B108" t="s">
+        <v>536</v>
+      </c>
+      <c r="C108" t="s">
+        <v>537</v>
+      </c>
+      <c r="D108" t="s">
+        <v>441</v>
+      </c>
+      <c r="E108" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>538</v>
+      </c>
+      <c r="B109" t="s">
+        <v>539</v>
+      </c>
+      <c r="C109" t="s">
+        <v>540</v>
+      </c>
+      <c r="D109" t="s">
+        <v>441</v>
+      </c>
+      <c r="E109" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>541</v>
+      </c>
+      <c r="B110" t="s">
+        <v>542</v>
+      </c>
+      <c r="C110" t="s">
+        <v>543</v>
+      </c>
+      <c r="D110" t="s">
+        <v>441</v>
+      </c>
+      <c r="E110" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>544</v>
+      </c>
+      <c r="B111" t="s">
+        <v>545</v>
+      </c>
+      <c r="C111" t="s">
+        <v>546</v>
+      </c>
+      <c r="D111" t="s">
+        <v>441</v>
+      </c>
+      <c r="E111" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>547</v>
+      </c>
+      <c r="B112" t="s">
+        <v>548</v>
+      </c>
+      <c r="C112" t="s">
+        <v>549</v>
+      </c>
+      <c r="D112" t="s">
+        <v>441</v>
+      </c>
+      <c r="E112" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>550</v>
+      </c>
+      <c r="B113" t="s">
+        <v>551</v>
+      </c>
+      <c r="C113" t="s">
+        <v>552</v>
+      </c>
+      <c r="D113" t="s">
+        <v>441</v>
+      </c>
+      <c r="E113" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>553</v>
+      </c>
+      <c r="B114" t="s">
+        <v>554</v>
+      </c>
+      <c r="C114" t="s">
+        <v>555</v>
+      </c>
+      <c r="D114" t="s">
+        <v>441</v>
+      </c>
+      <c r="E114" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>556</v>
+      </c>
+      <c r="B115" t="s">
+        <v>557</v>
+      </c>
+      <c r="C115" t="s">
+        <v>558</v>
+      </c>
+      <c r="D115" t="s">
+        <v>441</v>
+      </c>
+      <c r="E115" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>559</v>
+      </c>
+      <c r="B116" t="s">
+        <v>560</v>
+      </c>
+      <c r="C116" t="s">
+        <v>561</v>
+      </c>
+      <c r="D116" t="s">
+        <v>441</v>
+      </c>
+      <c r="E116" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>562</v>
+      </c>
+      <c r="B117" t="s">
+        <v>563</v>
+      </c>
+      <c r="C117" t="s">
+        <v>564</v>
+      </c>
+      <c r="D117" t="s">
+        <v>441</v>
+      </c>
+      <c r="E117" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>565</v>
+      </c>
+      <c r="B118" t="s">
+        <v>566</v>
+      </c>
+      <c r="C118" t="s">
+        <v>567</v>
+      </c>
+      <c r="D118" t="s">
+        <v>441</v>
+      </c>
+      <c r="E118" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>568</v>
+      </c>
+      <c r="B119" t="s">
+        <v>569</v>
+      </c>
+      <c r="C119" t="s">
+        <v>570</v>
+      </c>
+      <c r="D119" t="s">
+        <v>441</v>
+      </c>
+      <c r="E119" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>571</v>
+      </c>
+      <c r="B120" t="s">
+        <v>572</v>
+      </c>
+      <c r="C120" t="s">
+        <v>573</v>
+      </c>
+      <c r="D120" t="s">
+        <v>441</v>
+      </c>
+      <c r="E120" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>574</v>
+      </c>
+      <c r="B121" t="s">
+        <v>575</v>
+      </c>
+      <c r="C121" t="s">
+        <v>576</v>
+      </c>
+      <c r="D121" t="s">
+        <v>441</v>
+      </c>
+      <c r="E121" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>577</v>
+      </c>
+      <c r="B122" t="s">
+        <v>578</v>
+      </c>
+      <c r="C122" t="s">
+        <v>579</v>
+      </c>
+      <c r="D122" t="s">
+        <v>441</v>
+      </c>
+      <c r="E122" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>580</v>
+      </c>
+      <c r="B123" t="s">
+        <v>581</v>
+      </c>
+      <c r="C123" t="s">
+        <v>582</v>
+      </c>
+      <c r="D123" t="s">
+        <v>441</v>
+      </c>
+      <c r="E123" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>583</v>
+      </c>
+      <c r="B124" t="s">
+        <v>584</v>
+      </c>
+      <c r="C124" t="s">
+        <v>585</v>
+      </c>
+      <c r="D124" t="s">
+        <v>441</v>
+      </c>
+      <c r="E124" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>586</v>
+      </c>
+      <c r="B125" t="s">
+        <v>587</v>
+      </c>
+      <c r="C125" t="s">
+        <v>588</v>
+      </c>
+      <c r="D125" t="s">
+        <v>441</v>
+      </c>
+      <c r="E125" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>589</v>
+      </c>
+      <c r="B126" t="s">
+        <v>590</v>
+      </c>
+      <c r="C126" t="s">
+        <v>591</v>
+      </c>
+      <c r="D126" t="s">
+        <v>441</v>
+      </c>
+      <c r="E126" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>592</v>
+      </c>
+      <c r="B127" t="s">
+        <v>593</v>
+      </c>
+      <c r="C127" t="s">
+        <v>594</v>
+      </c>
+      <c r="D127" t="s">
+        <v>441</v>
+      </c>
+      <c r="E127" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>595</v>
+      </c>
+      <c r="B128" t="s">
+        <v>596</v>
+      </c>
+      <c r="C128" t="s">
+        <v>597</v>
+      </c>
+      <c r="D128" t="s">
+        <v>441</v>
+      </c>
+      <c r="E128" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>598</v>
+      </c>
+      <c r="B129" t="s">
+        <v>599</v>
+      </c>
+      <c r="C129" t="s">
+        <v>600</v>
+      </c>
+      <c r="D129" t="s">
+        <v>441</v>
+      </c>
+      <c r="E129" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>601</v>
+      </c>
+      <c r="B130" t="s">
+        <v>602</v>
+      </c>
+      <c r="C130" t="s">
+        <v>603</v>
+      </c>
+      <c r="D130" t="s">
+        <v>441</v>
+      </c>
+      <c r="E130" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>604</v>
+      </c>
+      <c r="B131" t="s">
+        <v>605</v>
+      </c>
+      <c r="C131" t="s">
+        <v>606</v>
+      </c>
+      <c r="D131" t="s">
+        <v>441</v>
+      </c>
+      <c r="E131" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>607</v>
+      </c>
+      <c r="B132" t="s">
+        <v>370</v>
+      </c>
+      <c r="C132" t="s">
+        <v>608</v>
+      </c>
+      <c r="D132" t="s">
+        <v>441</v>
+      </c>
+      <c r="E132" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>609</v>
+      </c>
+      <c r="B133" t="s">
+        <v>610</v>
+      </c>
+      <c r="C133" t="s">
+        <v>611</v>
+      </c>
+      <c r="D133" t="s">
+        <v>441</v>
+      </c>
+      <c r="E133" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>612</v>
+      </c>
+      <c r="B134" t="s">
+        <v>613</v>
+      </c>
+      <c r="C134" t="s">
+        <v>614</v>
+      </c>
+      <c r="D134" t="s">
+        <v>441</v>
+      </c>
+      <c r="E134" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>615</v>
+      </c>
+      <c r="B135" t="s">
+        <v>616</v>
+      </c>
+      <c r="C135" t="s">
+        <v>617</v>
+      </c>
+      <c r="D135" t="s">
+        <v>441</v>
+      </c>
+      <c r="E135" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>618</v>
+      </c>
+      <c r="B136" t="s">
+        <v>619</v>
+      </c>
+      <c r="C136" t="s">
+        <v>620</v>
+      </c>
+      <c r="D136" t="s">
+        <v>441</v>
+      </c>
+      <c r="E136" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>621</v>
+      </c>
+      <c r="B137" t="s">
+        <v>622</v>
+      </c>
+      <c r="C137" t="s">
+        <v>623</v>
+      </c>
+      <c r="D137" t="s">
+        <v>441</v>
+      </c>
+      <c r="E137" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>624</v>
+      </c>
+      <c r="B138" t="s">
+        <v>625</v>
+      </c>
+      <c r="C138" t="s">
+        <v>626</v>
+      </c>
+      <c r="D138" t="s">
+        <v>441</v>
+      </c>
+      <c r="E138" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>627</v>
+      </c>
+      <c r="B139" t="s">
+        <v>628</v>
+      </c>
+      <c r="C139" t="s">
+        <v>629</v>
+      </c>
+      <c r="D139" t="s">
+        <v>441</v>
+      </c>
+      <c r="E139" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete SA-004 logical entiity definitions and data dictionary
</commit_message>
<xml_diff>
--- a/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
+++ b/Documentation/Formal/DOC-007 Business Discovery Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd01d60e8fdc72b3/Projects/Construction_Analytics_Platform/Documentation/Formal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="141" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{913AA438-1A64-45F0-9FD5-12D0AFEF00BA}"/>
+  <xr:revisionPtr revIDLastSave="183" documentId="8_{A16E292A-D5FD-4100-B9C8-DBE701A8725A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF574556-5BA4-4E94-BF61-6055A5BB6F9E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15900" activeTab="2" xr2:uid="{8CD3C967-02BD-42FB-BAFC-E9F1B6D02552}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="749">
   <si>
     <t>KPI</t>
   </si>
@@ -1934,6 +1934,363 @@
   </si>
   <si>
     <t>The solution shall lock configuration values that affect historical comparability after implementation or require a controlled conversion process before changing them.</t>
+  </si>
+  <si>
+    <t>FR-139</t>
+  </si>
+  <si>
+    <t>Lean Analytics Scope</t>
+  </si>
+  <si>
+    <t>The sample database shall be designed as a construction analytics portfolio database rather than an operational ERP system.</t>
+  </si>
+  <si>
+    <t>SA-004</t>
+  </si>
+  <si>
+    <t>FR-140</t>
+  </si>
+  <si>
+    <t>Job Identifiers</t>
+  </si>
+  <si>
+    <t>The Job entity shall store an internal Job ID and a source-system Job Number.</t>
+  </si>
+  <si>
+    <t>FR-141</t>
+  </si>
+  <si>
+    <t>Job Reopening</t>
+  </si>
+  <si>
+    <t>A reopened Job shall return to Active and retain a Reopened Flag and Most Recent Reopened Date.</t>
+  </si>
+  <si>
+    <t>FR-142</t>
+  </si>
+  <si>
+    <t>Job Quote Lineage</t>
+  </si>
+  <si>
+    <t>The system shall preserve the accepted Quotes and Bid Budgets that collectively form the original Job.</t>
+  </si>
+  <si>
+    <t>FR-143</t>
+  </si>
+  <si>
+    <t>Single Component Budget</t>
+  </si>
+  <si>
+    <t>Each Job Component shall have no more than one Component Budget.</t>
+  </si>
+  <si>
+    <t>FR-144</t>
+  </si>
+  <si>
+    <t>Budget Detail Grain</t>
+  </si>
+  <si>
+    <t>Budget Detail shall be stored by Component Budget, Cost Code, Phase, and Cost Type.</t>
+  </si>
+  <si>
+    <t>FR-145</t>
+  </si>
+  <si>
+    <t>Optional Budget Quantity</t>
+  </si>
+  <si>
+    <t>Budget Quantity and Unit of Measure shall be optional for lump-sum budget lines.</t>
+  </si>
+  <si>
+    <t>FR-146</t>
+  </si>
+  <si>
+    <t>Budget Total Calculation</t>
+  </si>
+  <si>
+    <t>Budget Total Cost shall be calculated from Quantity and Unit Cost when both values exist.</t>
+  </si>
+  <si>
+    <t>FR-147</t>
+  </si>
+  <si>
+    <t>Stored Revenue Allocation</t>
+  </si>
+  <si>
+    <t>Calculated revenue allocation shall be stored at Budget Detail level.</t>
+  </si>
+  <si>
+    <t>FR-148</t>
+  </si>
+  <si>
+    <t>Original Budget Detail values shall remain unchanged after creation.</t>
+  </si>
+  <si>
+    <t>FR-149</t>
+  </si>
+  <si>
+    <t>Quantity, Unit Cost, and Total Cost changes shall be stored as Budget Adjustment records.</t>
+  </si>
+  <si>
+    <t>FR-150</t>
+  </si>
+  <si>
+    <t>Cost Code Structure</t>
+  </si>
+  <si>
+    <t>Cost Code shall use the numeric business code as its identifier and store a separate name and description.</t>
+  </si>
+  <si>
+    <t>FR-151</t>
+  </si>
+  <si>
+    <t>Shared Cost Codes</t>
+  </si>
+  <si>
+    <t>Cost Codes shall be available across all divisions.</t>
+  </si>
+  <si>
+    <t>FR-152</t>
+  </si>
+  <si>
+    <t>Phase Structure</t>
+  </si>
+  <si>
+    <t>Phase shall store Phase Code, Phase Name, and Description.</t>
+  </si>
+  <si>
+    <t>FR-153</t>
+  </si>
+  <si>
+    <t>Default Production Phases</t>
+  </si>
+  <si>
+    <t>Phases 900 and 905 shall be available for production and travel activity.</t>
+  </si>
+  <si>
+    <t>FR-154</t>
+  </si>
+  <si>
+    <t>Warranty Phases</t>
+  </si>
+  <si>
+    <t>Phases 950 and 955 shall be used only when warranty activity occurs.</t>
+  </si>
+  <si>
+    <t>FR-155</t>
+  </si>
+  <si>
+    <t>Employee Identifier</t>
+  </si>
+  <si>
+    <t>Employee shall use the source-system Employee ID as its identifier.</t>
+  </si>
+  <si>
+    <t>FR-156</t>
+  </si>
+  <si>
+    <t>Employee Analytics Attributes</t>
+  </si>
+  <si>
+    <t>Employee shall store only attributes required for operational analytics and shall exclude date of birth and home address.</t>
+  </si>
+  <si>
+    <t>FR-157</t>
+  </si>
+  <si>
+    <t>Planning Crews</t>
+  </si>
+  <si>
+    <t>Crew shall support planning, while daily work groups shall be derived from labor records.</t>
+  </si>
+  <si>
+    <t>FR-158</t>
+  </si>
+  <si>
+    <t>Labor Rate Codes</t>
+  </si>
+  <si>
+    <t>An Employee shall support multiple labor Rate Codes with Regular Time, Overtime, and Double Time rates.</t>
+  </si>
+  <si>
+    <t>FR-159</t>
+  </si>
+  <si>
+    <t>Time Entry Grain</t>
+  </si>
+  <si>
+    <t>Employee Time Entry shall identify Employee, Work Date, Job, Cost Code, Phase, Rate Code, and Foreman.</t>
+  </si>
+  <si>
+    <t>FR-160</t>
+  </si>
+  <si>
+    <t>Daily Work Group</t>
+  </si>
+  <si>
+    <t>Daily work groups shall be derived by Job, Work Date, and Foreman.</t>
+  </si>
+  <si>
+    <t>FR-161</t>
+  </si>
+  <si>
+    <t>Estimated Labor Cost</t>
+  </si>
+  <si>
+    <t>Same-day estimated labor cost shall use Time Entry hours and the applicable Employee labor rates.</t>
+  </si>
+  <si>
+    <t>FR-162</t>
+  </si>
+  <si>
+    <t>Separate Burden</t>
+  </si>
+  <si>
+    <t>Estimated Burden shall remain separate from Labor under Cost Type B.</t>
+  </si>
+  <si>
+    <t>FR-163</t>
+  </si>
+  <si>
+    <t>Equipment Identifier</t>
+  </si>
+  <si>
+    <t>Equipment shall use an internal Equipment ID and retain a business-facing Equipment Number.</t>
+  </si>
+  <si>
+    <t>FR-164</t>
+  </si>
+  <si>
+    <t>Equipment Current Rate</t>
+  </si>
+  <si>
+    <t>Equipment shall store one current hourly rate, and Equipment Usage shall retain the applied rate.</t>
+  </si>
+  <si>
+    <t>FR-165</t>
+  </si>
+  <si>
+    <t>Material Identifier</t>
+  </si>
+  <si>
+    <t>Material shall use an internal Material ID and may store an optional Material Code.</t>
+  </si>
+  <si>
+    <t>FR-166</t>
+  </si>
+  <si>
+    <t>Material Categories</t>
+  </si>
+  <si>
+    <t>The system shall support extensible Material Categories beginning with Asphalt, Concrete, Sealer, Crackfill Rubber, Paint, General Materials, and Other.</t>
+  </si>
+  <si>
+    <t>FR-167</t>
+  </si>
+  <si>
+    <t>Material Usage Cost</t>
+  </si>
+  <si>
+    <t>Material Usage Total Cost shall equal Quantity multiplied by Applied Unit Cost.</t>
+  </si>
+  <si>
+    <t>FR-168</t>
+  </si>
+  <si>
+    <t>Vendor Identifier</t>
+  </si>
+  <si>
+    <t>Vendor shall use an internal Vendor ID.</t>
+  </si>
+  <si>
+    <t>FR-169</t>
+  </si>
+  <si>
+    <t>Analytical PO Commitments</t>
+  </si>
+  <si>
+    <t>Purchase Order Commitment shall provide ordered, committed, invoiced, and open-commitment values at PO-line level.</t>
+  </si>
+  <si>
+    <t>FR-170</t>
+  </si>
+  <si>
+    <t>Posted Job Cost shall be authoritative for final financial cost.</t>
+  </si>
+  <si>
+    <t>FR-171</t>
+  </si>
+  <si>
+    <t>Job-Level Billing</t>
+  </si>
+  <si>
+    <t>Customer Billing shall be stored at Job level without Cost Code or Job Component allocation.</t>
+  </si>
+  <si>
+    <t>FR-172</t>
+  </si>
+  <si>
+    <t>Daily Production</t>
+  </si>
+  <si>
+    <t>Daily Production shall store production quantity by Work Date, Job, Cost Code, and Foreman.</t>
+  </si>
+  <si>
+    <t>FR-173</t>
+  </si>
+  <si>
+    <t>Operational Delays</t>
+  </si>
+  <si>
+    <t>Operational Delay shall store Delay Type and Delay Hours by Work Date and Job with optional Cost Code and Foreman.</t>
+  </si>
+  <si>
+    <t>FR-174</t>
+  </si>
+  <si>
+    <t>The system shall retain one current Forecast per Job.</t>
+  </si>
+  <si>
+    <t>FR-175</t>
+  </si>
+  <si>
+    <t>Forecast Detail shall support Cost Code and optional Cost Type detail.</t>
+  </si>
+  <si>
+    <t>FR-176</t>
+  </si>
+  <si>
+    <t>WIP Snapshots</t>
+  </si>
+  <si>
+    <t>The system shall preserve Weekly and Month-End WIP Snapshots.</t>
+  </si>
+  <si>
+    <t>FR-177</t>
+  </si>
+  <si>
+    <t>Estimate Replacement</t>
+  </si>
+  <si>
+    <t>When Posted Job Cost exists for the same Job, Work Date, Cost Code, Phase, and Cost Type, posted cost shall replace estimated operational cost for financial reporting.</t>
+  </si>
+  <si>
+    <t>FR-178</t>
+  </si>
+  <si>
+    <t>Operational Quantity Authority</t>
+  </si>
+  <si>
+    <t>Operational hours and quantities shall remain available for production and utilization analysis after financial cost posts.</t>
+  </si>
+  <si>
+    <t>FR-179</t>
+  </si>
+  <si>
+    <t>Deferred ERP Features</t>
+  </si>
+  <si>
+    <t>Full payroll, supplier workflow, approval routing, multi-company configuration, and detailed matching shall be deferred from the sample database.</t>
   </si>
 </sst>
 </file>
@@ -3428,7 +3785,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{979FD651-F2D4-4BEE-84B1-39B645FFAE94}">
-  <dimension ref="A1:E139"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
@@ -5798,6 +6155,703 @@
         <v>441</v>
       </c>
       <c r="E139" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>630</v>
+      </c>
+      <c r="B140" t="s">
+        <v>631</v>
+      </c>
+      <c r="C140" t="s">
+        <v>632</v>
+      </c>
+      <c r="D140" t="s">
+        <v>633</v>
+      </c>
+      <c r="E140" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>634</v>
+      </c>
+      <c r="B141" t="s">
+        <v>635</v>
+      </c>
+      <c r="C141" t="s">
+        <v>636</v>
+      </c>
+      <c r="D141" t="s">
+        <v>633</v>
+      </c>
+      <c r="E141" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>637</v>
+      </c>
+      <c r="B142" t="s">
+        <v>638</v>
+      </c>
+      <c r="C142" t="s">
+        <v>639</v>
+      </c>
+      <c r="D142" t="s">
+        <v>633</v>
+      </c>
+      <c r="E142" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>640</v>
+      </c>
+      <c r="B143" t="s">
+        <v>641</v>
+      </c>
+      <c r="C143" t="s">
+        <v>642</v>
+      </c>
+      <c r="D143" t="s">
+        <v>633</v>
+      </c>
+      <c r="E143" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>643</v>
+      </c>
+      <c r="B144" t="s">
+        <v>644</v>
+      </c>
+      <c r="C144" t="s">
+        <v>645</v>
+      </c>
+      <c r="D144" t="s">
+        <v>633</v>
+      </c>
+      <c r="E144" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>646</v>
+      </c>
+      <c r="B145" t="s">
+        <v>647</v>
+      </c>
+      <c r="C145" t="s">
+        <v>648</v>
+      </c>
+      <c r="D145" t="s">
+        <v>633</v>
+      </c>
+      <c r="E145" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>649</v>
+      </c>
+      <c r="B146" t="s">
+        <v>650</v>
+      </c>
+      <c r="C146" t="s">
+        <v>651</v>
+      </c>
+      <c r="D146" t="s">
+        <v>633</v>
+      </c>
+      <c r="E146" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>652</v>
+      </c>
+      <c r="B147" t="s">
+        <v>653</v>
+      </c>
+      <c r="C147" t="s">
+        <v>654</v>
+      </c>
+      <c r="D147" t="s">
+        <v>633</v>
+      </c>
+      <c r="E147" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>655</v>
+      </c>
+      <c r="B148" t="s">
+        <v>656</v>
+      </c>
+      <c r="C148" t="s">
+        <v>657</v>
+      </c>
+      <c r="D148" t="s">
+        <v>633</v>
+      </c>
+      <c r="E148" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>658</v>
+      </c>
+      <c r="B149" t="s">
+        <v>220</v>
+      </c>
+      <c r="C149" t="s">
+        <v>659</v>
+      </c>
+      <c r="D149" t="s">
+        <v>633</v>
+      </c>
+      <c r="E149" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>660</v>
+      </c>
+      <c r="B150" t="s">
+        <v>229</v>
+      </c>
+      <c r="C150" t="s">
+        <v>661</v>
+      </c>
+      <c r="D150" t="s">
+        <v>633</v>
+      </c>
+      <c r="E150" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>662</v>
+      </c>
+      <c r="B151" t="s">
+        <v>663</v>
+      </c>
+      <c r="C151" t="s">
+        <v>664</v>
+      </c>
+      <c r="D151" t="s">
+        <v>633</v>
+      </c>
+      <c r="E151" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>665</v>
+      </c>
+      <c r="B152" t="s">
+        <v>666</v>
+      </c>
+      <c r="C152" t="s">
+        <v>667</v>
+      </c>
+      <c r="D152" t="s">
+        <v>633</v>
+      </c>
+      <c r="E152" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>668</v>
+      </c>
+      <c r="B153" t="s">
+        <v>669</v>
+      </c>
+      <c r="C153" t="s">
+        <v>670</v>
+      </c>
+      <c r="D153" t="s">
+        <v>633</v>
+      </c>
+      <c r="E153" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>671</v>
+      </c>
+      <c r="B154" t="s">
+        <v>672</v>
+      </c>
+      <c r="C154" t="s">
+        <v>673</v>
+      </c>
+      <c r="D154" t="s">
+        <v>633</v>
+      </c>
+      <c r="E154" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>674</v>
+      </c>
+      <c r="B155" t="s">
+        <v>675</v>
+      </c>
+      <c r="C155" t="s">
+        <v>676</v>
+      </c>
+      <c r="D155" t="s">
+        <v>633</v>
+      </c>
+      <c r="E155" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>677</v>
+      </c>
+      <c r="B156" t="s">
+        <v>678</v>
+      </c>
+      <c r="C156" t="s">
+        <v>679</v>
+      </c>
+      <c r="D156" t="s">
+        <v>633</v>
+      </c>
+      <c r="E156" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>680</v>
+      </c>
+      <c r="B157" t="s">
+        <v>681</v>
+      </c>
+      <c r="C157" t="s">
+        <v>682</v>
+      </c>
+      <c r="D157" t="s">
+        <v>633</v>
+      </c>
+      <c r="E157" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>683</v>
+      </c>
+      <c r="B158" t="s">
+        <v>684</v>
+      </c>
+      <c r="C158" t="s">
+        <v>685</v>
+      </c>
+      <c r="D158" t="s">
+        <v>633</v>
+      </c>
+      <c r="E158" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>686</v>
+      </c>
+      <c r="B159" t="s">
+        <v>687</v>
+      </c>
+      <c r="C159" t="s">
+        <v>688</v>
+      </c>
+      <c r="D159" t="s">
+        <v>633</v>
+      </c>
+      <c r="E159" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>689</v>
+      </c>
+      <c r="B160" t="s">
+        <v>690</v>
+      </c>
+      <c r="C160" t="s">
+        <v>691</v>
+      </c>
+      <c r="D160" t="s">
+        <v>633</v>
+      </c>
+      <c r="E160" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>692</v>
+      </c>
+      <c r="B161" t="s">
+        <v>693</v>
+      </c>
+      <c r="C161" t="s">
+        <v>694</v>
+      </c>
+      <c r="D161" t="s">
+        <v>633</v>
+      </c>
+      <c r="E161" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>695</v>
+      </c>
+      <c r="B162" t="s">
+        <v>696</v>
+      </c>
+      <c r="C162" t="s">
+        <v>697</v>
+      </c>
+      <c r="D162" t="s">
+        <v>633</v>
+      </c>
+      <c r="E162" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>698</v>
+      </c>
+      <c r="B163" t="s">
+        <v>699</v>
+      </c>
+      <c r="C163" t="s">
+        <v>700</v>
+      </c>
+      <c r="D163" t="s">
+        <v>633</v>
+      </c>
+      <c r="E163" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>701</v>
+      </c>
+      <c r="B164" t="s">
+        <v>702</v>
+      </c>
+      <c r="C164" t="s">
+        <v>703</v>
+      </c>
+      <c r="D164" t="s">
+        <v>633</v>
+      </c>
+      <c r="E164" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>704</v>
+      </c>
+      <c r="B165" t="s">
+        <v>705</v>
+      </c>
+      <c r="C165" t="s">
+        <v>706</v>
+      </c>
+      <c r="D165" t="s">
+        <v>633</v>
+      </c>
+      <c r="E165" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>707</v>
+      </c>
+      <c r="B166" t="s">
+        <v>708</v>
+      </c>
+      <c r="C166" t="s">
+        <v>709</v>
+      </c>
+      <c r="D166" t="s">
+        <v>633</v>
+      </c>
+      <c r="E166" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>710</v>
+      </c>
+      <c r="B167" t="s">
+        <v>711</v>
+      </c>
+      <c r="C167" t="s">
+        <v>712</v>
+      </c>
+      <c r="D167" t="s">
+        <v>633</v>
+      </c>
+      <c r="E167" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>713</v>
+      </c>
+      <c r="B168" t="s">
+        <v>714</v>
+      </c>
+      <c r="C168" t="s">
+        <v>715</v>
+      </c>
+      <c r="D168" t="s">
+        <v>633</v>
+      </c>
+      <c r="E168" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>716</v>
+      </c>
+      <c r="B169" t="s">
+        <v>717</v>
+      </c>
+      <c r="C169" t="s">
+        <v>718</v>
+      </c>
+      <c r="D169" t="s">
+        <v>633</v>
+      </c>
+      <c r="E169" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>719</v>
+      </c>
+      <c r="B170" t="s">
+        <v>720</v>
+      </c>
+      <c r="C170" t="s">
+        <v>721</v>
+      </c>
+      <c r="D170" t="s">
+        <v>633</v>
+      </c>
+      <c r="E170" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>722</v>
+      </c>
+      <c r="B171" t="s">
+        <v>533</v>
+      </c>
+      <c r="C171" t="s">
+        <v>723</v>
+      </c>
+      <c r="D171" t="s">
+        <v>633</v>
+      </c>
+      <c r="E171" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>724</v>
+      </c>
+      <c r="B172" t="s">
+        <v>725</v>
+      </c>
+      <c r="C172" t="s">
+        <v>726</v>
+      </c>
+      <c r="D172" t="s">
+        <v>633</v>
+      </c>
+      <c r="E172" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>727</v>
+      </c>
+      <c r="B173" t="s">
+        <v>728</v>
+      </c>
+      <c r="C173" t="s">
+        <v>729</v>
+      </c>
+      <c r="D173" t="s">
+        <v>633</v>
+      </c>
+      <c r="E173" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>730</v>
+      </c>
+      <c r="B174" t="s">
+        <v>731</v>
+      </c>
+      <c r="C174" t="s">
+        <v>732</v>
+      </c>
+      <c r="D174" t="s">
+        <v>633</v>
+      </c>
+      <c r="E174" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>733</v>
+      </c>
+      <c r="B175" t="s">
+        <v>593</v>
+      </c>
+      <c r="C175" t="s">
+        <v>734</v>
+      </c>
+      <c r="D175" t="s">
+        <v>633</v>
+      </c>
+      <c r="E175" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>735</v>
+      </c>
+      <c r="B176" t="s">
+        <v>421</v>
+      </c>
+      <c r="C176" t="s">
+        <v>736</v>
+      </c>
+      <c r="D176" t="s">
+        <v>633</v>
+      </c>
+      <c r="E176" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>737</v>
+      </c>
+      <c r="B177" t="s">
+        <v>738</v>
+      </c>
+      <c r="C177" t="s">
+        <v>739</v>
+      </c>
+      <c r="D177" t="s">
+        <v>633</v>
+      </c>
+      <c r="E177" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>740</v>
+      </c>
+      <c r="B178" t="s">
+        <v>741</v>
+      </c>
+      <c r="C178" t="s">
+        <v>742</v>
+      </c>
+      <c r="D178" t="s">
+        <v>633</v>
+      </c>
+      <c r="E178" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>743</v>
+      </c>
+      <c r="B179" t="s">
+        <v>744</v>
+      </c>
+      <c r="C179" t="s">
+        <v>745</v>
+      </c>
+      <c r="D179" t="s">
+        <v>633</v>
+      </c>
+      <c r="E179" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>746</v>
+      </c>
+      <c r="B180" t="s">
+        <v>747</v>
+      </c>
+      <c r="C180" t="s">
+        <v>748</v>
+      </c>
+      <c r="D180" t="s">
+        <v>633</v>
+      </c>
+      <c r="E180" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>